<commit_message>
Add Manual MSISDN Entry to the Number Selection step
A card below the existing Free/Star number grid lets an agent reserve any
MSISDN not in the seeded inventory: a full +974-prefixed 8-digit number,
validated the same way GuidedContactStep validates a Qatar local number,
with the "Reserve Custom Number" button disabled until the format is
valid. Checks the entered number against numbers.json so a seeded
Blocked/Reserved number is rejected with the same clarity as picking it
from the grid would be, instead of silently double-booking it.

Shared MsisdnPicker component — this is available everywhere Number
Selection already appears (New Postpaid, Fixed Line, FWA), not just one
wizard.

Also updates the test-data reference workbook with the seeded MSISDN
inventory and how to exercise this feature's valid/blocked/malformed
paths.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/vfq-dxp-app/reference/VFQ_DXP_Test_Data_Reference.xlsx
+++ b/vfq-dxp-app/reference/VFQ_DXP_Test_Data_Reference.xlsx
@@ -18,7 +18,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bulk Notes" sheetId="9" state="visible" r:id="rId9"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Leads (Sales)" sheetId="10" state="visible" r:id="rId10"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Postpaid Plans &amp; Discounts" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Verification Codes" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Number Selection" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Verification Codes" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -494,7 +495,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D15"/>
+  <dimension ref="A1:D16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -650,10 +651,22 @@
     <row r="15" ht="30" customHeight="1">
       <c r="A15" s="4" t="inlineStr">
         <is>
+          <t>Number Selection</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>Seeded MSISDN inventory plus how to test the Manual MSISDN Entry card's valid/blocked/malformed paths.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="30" customHeight="1">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
           <t>Verification Codes</t>
         </is>
       </c>
-      <c r="B15" s="5" t="inlineStr">
+      <c r="B16" s="5" t="inlineStr">
         <is>
           <t>The demo password and OTP/verification code used everywhere a code is required (password reset, MFA, change password).</t>
         </is>
@@ -1182,6 +1195,155 @@
 </file>
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>Number Selection</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>public/mock-data/numbers.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="45" customHeight="1">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>The Number Selection step (New Postpaid/Fixed Line/FWA wizards) also has a "Manual MSISDN Entry" card below the grid for reserving any MSISDN not in the seeded inventory below — type a full +974-prefixed 8-digit number (e.g. +974 3300 9999) and click "Reserve Custom Number". To test its rejection paths: type +97433001003 (seeded as Blocked below) to see the "already blocked" error, or an incomplete/malformed number to see the format error.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="28" customHeight="1">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>MSISDN</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>Price (QAR)</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>Value Tier</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="30" customHeight="1">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>+97433001001</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>Reserved</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="30" customHeight="1">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>+97433001002</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>Star</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>AVAILABLE</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="n">
+        <v>500</v>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="30" customHeight="1">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>+97433001003</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A4:F4"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Re-save VFQ_DXP_Test_Data_Reference.xlsx (no content changes)
Cell-by-cell diff against HEAD across every sheet shows zero content
differences — Excel metadata only, from the file being open/re-saved
locally (a lock file is present alongside it).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/vfq-dxp-app/reference/VFQ_DXP_Test_Data_Reference.xlsx
+++ b/vfq-dxp-app/reference/VFQ_DXP_Test_Data_Reference.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/parithimalsaravanan/claude-projects/vfq/vfq-dxp-app/reference/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4795B1F2-9AF3-F94B-94B9-7BE5417B2B5A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92ACBFF3-6A36-BE4F-B905-DCD3808E2C99}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="21680" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-38400" yWindow="2300" windowWidth="38400" windowHeight="23400" firstSheet="4" activeTab="14" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Start Here" sheetId="1" r:id="rId1"/>
@@ -1570,21 +1570,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -1593,17 +1584,56 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
+      <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1910,26 +1940,26 @@
   <dimension ref="A1:D19"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="26" style="4" customWidth="1"/>
-    <col min="2" max="2" width="95" style="4" customWidth="1"/>
-    <col min="3" max="16384" width="8.83203125" style="4"/>
+    <col min="1" max="1" width="26" style="2" customWidth="1"/>
+    <col min="2" max="2" width="95" style="2" customWidth="1"/>
+    <col min="3" max="16384" width="8.83203125" style="2"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="26" x14ac:dyDescent="0.2">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3"/>
-      <c r="C1" s="3"/>
-      <c r="D1" s="3"/>
+      <c r="B1" s="6"/>
+      <c r="C1" s="6"/>
+      <c r="D1" s="6"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A2" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="3"/>
-      <c r="C2" s="3"/>
-      <c r="D2" s="3"/>
+      <c r="B2" s="6"/>
+      <c r="C2" s="6"/>
+      <c r="D2" s="6"/>
     </row>
     <row r="4" spans="1:4" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
@@ -1940,122 +1970,122 @@
       </c>
     </row>
     <row r="5" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="6" t="s">
+      <c r="A5" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="7" t="s">
+      <c r="B5" s="4" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="6" t="s">
+      <c r="A6" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="7" t="s">
+      <c r="B6" s="4" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="6" t="s">
+      <c r="A7" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B7" s="7" t="s">
+      <c r="B7" s="4" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="6" t="s">
+      <c r="A8" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="B8" s="7" t="s">
+      <c r="B8" s="4" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="6" t="s">
+      <c r="A9" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="B9" s="7" t="s">
+      <c r="B9" s="4" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="6" t="s">
+      <c r="A10" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="B10" s="7" t="s">
+      <c r="B10" s="4" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="6" t="s">
+      <c r="A11" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="B11" s="7" t="s">
+      <c r="B11" s="4" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="12" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="6" t="s">
+      <c r="A12" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="B12" s="7" t="s">
+      <c r="B12" s="4" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="13" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="6" t="s">
+      <c r="A13" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="B13" s="7" t="s">
+      <c r="B13" s="4" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="14" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="6" t="s">
+      <c r="A14" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="B14" s="7" t="s">
+      <c r="B14" s="4" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="15" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="6" t="s">
+      <c r="A15" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="B15" s="7" t="s">
+      <c r="B15" s="4" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="16" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="6" t="s">
+      <c r="A16" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="B16" s="7" t="s">
+      <c r="B16" s="4" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="17" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="6" t="s">
+      <c r="A17" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="B17" s="7" t="s">
+      <c r="B17" s="4" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="18" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="6" t="s">
+      <c r="A18" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="B18" s="7" t="s">
+      <c r="B18" s="4" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="19" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="6" t="s">
+      <c r="A19" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="B19" s="7" t="s">
+      <c r="B19" s="4" t="s">
         <v>33</v>
       </c>
     </row>
@@ -2076,91 +2106,91 @@
   <dimension ref="A1:F6"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="14" style="4" customWidth="1"/>
-    <col min="2" max="2" width="18" style="4" customWidth="1"/>
-    <col min="3" max="4" width="20" style="4" customWidth="1"/>
-    <col min="5" max="5" width="18" style="4" customWidth="1"/>
-    <col min="6" max="6" width="16" style="4" customWidth="1"/>
-    <col min="7" max="16384" width="8.83203125" style="4"/>
+    <col min="1" max="1" width="14" style="15" customWidth="1"/>
+    <col min="2" max="2" width="18" style="15" customWidth="1"/>
+    <col min="3" max="4" width="20" style="15" customWidth="1"/>
+    <col min="5" max="5" width="18" style="15" customWidth="1"/>
+    <col min="6" max="6" width="16" style="15" customWidth="1"/>
+    <col min="7" max="16384" width="8.83203125" style="2"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="21" x14ac:dyDescent="0.2">
-      <c r="A1" s="8" t="s">
+      <c r="A1" s="16" t="s">
         <v>331</v>
       </c>
-      <c r="B1" s="3"/>
-      <c r="C1" s="3"/>
-      <c r="D1" s="3"/>
-      <c r="E1" s="3"/>
-      <c r="F1" s="3"/>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="17"/>
+      <c r="F1" s="17"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A2" s="5" t="s">
+      <c r="A2" s="18" t="s">
         <v>332</v>
       </c>
-      <c r="B2" s="3"/>
-      <c r="C2" s="3"/>
-      <c r="D2" s="3"/>
-      <c r="E2" s="3"/>
-      <c r="F2" s="3"/>
+      <c r="B2" s="17"/>
+      <c r="C2" s="17"/>
+      <c r="D2" s="17"/>
+      <c r="E2" s="17"/>
+      <c r="F2" s="17"/>
     </row>
     <row r="4" spans="1:6" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="1" t="s">
+      <c r="A4" s="13" t="s">
         <v>333</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B4" s="13" t="s">
         <v>334</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="C4" s="13" t="s">
         <v>167</v>
       </c>
-      <c r="D4" s="1" t="s">
+      <c r="D4" s="13" t="s">
         <v>335</v>
       </c>
-      <c r="E4" s="1" t="s">
+      <c r="E4" s="13" t="s">
         <v>101</v>
       </c>
-      <c r="F4" s="1" t="s">
+      <c r="F4" s="13" t="s">
         <v>336</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="7" t="s">
+      <c r="A5" s="14" t="s">
         <v>337</v>
       </c>
-      <c r="B5" s="7" t="s">
+      <c r="B5" s="14" t="s">
         <v>338</v>
       </c>
-      <c r="C5" s="7" t="s">
+      <c r="C5" s="14" t="s">
         <v>339</v>
       </c>
-      <c r="D5" s="7" t="s">
+      <c r="D5" s="14" t="s">
         <v>340</v>
       </c>
-      <c r="E5" s="7" t="s">
+      <c r="E5" s="14" t="s">
         <v>90</v>
       </c>
-      <c r="F5" s="7" t="s">
+      <c r="F5" s="14" t="s">
         <v>341</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="7" t="s">
+      <c r="A6" s="14" t="s">
         <v>342</v>
       </c>
-      <c r="B6" s="7" t="s">
+      <c r="B6" s="14" t="s">
         <v>343</v>
       </c>
-      <c r="C6" s="7" t="s">
+      <c r="C6" s="14" t="s">
         <v>344</v>
       </c>
-      <c r="D6" s="7" t="s">
+      <c r="D6" s="14" t="s">
         <v>345</v>
       </c>
-      <c r="E6" s="7" t="s">
+      <c r="E6" s="14" t="s">
         <v>346</v>
       </c>
-      <c r="F6" s="7" t="s">
+      <c r="F6" s="14" t="s">
         <v>90</v>
       </c>
     </row>
@@ -2181,310 +2211,310 @@
   <dimension ref="A1:G23"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="14" style="4" customWidth="1"/>
-    <col min="2" max="2" width="18" style="4" customWidth="1"/>
-    <col min="3" max="3" width="20" style="4" customWidth="1"/>
-    <col min="4" max="4" width="10" style="4" customWidth="1"/>
-    <col min="5" max="5" width="44" style="4" customWidth="1"/>
-    <col min="6" max="6" width="16" style="4" customWidth="1"/>
-    <col min="7" max="7" width="12" style="4" customWidth="1"/>
-    <col min="8" max="16384" width="8.83203125" style="4"/>
+    <col min="1" max="1" width="14" style="15" customWidth="1"/>
+    <col min="2" max="2" width="18" style="15" customWidth="1"/>
+    <col min="3" max="3" width="20" style="15" customWidth="1"/>
+    <col min="4" max="4" width="10" style="15" customWidth="1"/>
+    <col min="5" max="5" width="44" style="15" customWidth="1"/>
+    <col min="6" max="6" width="16" style="15" customWidth="1"/>
+    <col min="7" max="7" width="12" style="15" customWidth="1"/>
+    <col min="8" max="16384" width="8.83203125" style="2"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="21" x14ac:dyDescent="0.2">
-      <c r="A1" s="8" t="s">
+      <c r="A1" s="16" t="s">
         <v>22</v>
       </c>
-      <c r="B1" s="3"/>
-      <c r="C1" s="3"/>
-      <c r="D1" s="3"/>
-      <c r="E1" s="3"/>
-      <c r="F1" s="3"/>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="17"/>
+      <c r="F1" s="17"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A2" s="5" t="s">
+      <c r="A2" s="18" t="s">
         <v>347</v>
       </c>
-      <c r="B2" s="3"/>
-      <c r="C2" s="3"/>
-      <c r="D2" s="3"/>
-      <c r="E2" s="3"/>
-      <c r="F2" s="3"/>
+      <c r="B2" s="17"/>
+      <c r="C2" s="17"/>
+      <c r="D2" s="17"/>
+      <c r="E2" s="17"/>
+      <c r="F2" s="17"/>
     </row>
     <row r="4" spans="1:7" ht="45" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="9" t="s">
+      <c r="A4" s="19" t="s">
         <v>348</v>
       </c>
-      <c r="B4" s="3"/>
-      <c r="C4" s="3"/>
-      <c r="D4" s="3"/>
-      <c r="E4" s="3"/>
-      <c r="F4" s="3"/>
+      <c r="B4" s="17"/>
+      <c r="C4" s="17"/>
+      <c r="D4" s="17"/>
+      <c r="E4" s="17"/>
+      <c r="F4" s="17"/>
     </row>
     <row r="6" spans="1:7" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="1" t="s">
+      <c r="A6" s="13" t="s">
         <v>349</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="B6" s="13" t="s">
         <v>350</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="C6" s="13" t="s">
         <v>351</v>
       </c>
-      <c r="D6" s="1" t="s">
+      <c r="D6" s="13" t="s">
         <v>272</v>
       </c>
-      <c r="E6" s="1" t="s">
+      <c r="E6" s="13" t="s">
         <v>352</v>
       </c>
-      <c r="F6" s="1" t="s">
+      <c r="F6" s="13" t="s">
         <v>353</v>
       </c>
-      <c r="G6" s="1" t="s">
+      <c r="G6" s="13" t="s">
         <v>354</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="7" t="s">
+      <c r="A7" s="14" t="s">
         <v>355</v>
       </c>
-      <c r="B7" s="7" t="s">
+      <c r="B7" s="14" t="s">
         <v>356</v>
       </c>
-      <c r="C7" s="7">
+      <c r="C7" s="14">
         <v>250</v>
       </c>
-      <c r="D7" s="7">
+      <c r="D7" s="14">
         <v>30</v>
       </c>
-      <c r="E7" s="7" t="s">
+      <c r="E7" s="14" t="s">
         <v>357</v>
       </c>
-      <c r="F7" s="7" t="s">
+      <c r="F7" s="14" t="s">
         <v>358</v>
       </c>
-      <c r="G7" s="7"/>
+      <c r="G7" s="14"/>
     </row>
     <row r="8" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="7" t="s">
+      <c r="A8" s="14" t="s">
         <v>359</v>
       </c>
-      <c r="B8" s="7" t="s">
+      <c r="B8" s="14" t="s">
         <v>360</v>
       </c>
-      <c r="C8" s="7">
+      <c r="C8" s="14">
         <v>350</v>
       </c>
-      <c r="D8" s="7">
+      <c r="D8" s="14">
         <v>100</v>
       </c>
-      <c r="E8" s="7" t="s">
+      <c r="E8" s="14" t="s">
         <v>357</v>
       </c>
-      <c r="F8" s="7" t="s">
+      <c r="F8" s="14" t="s">
         <v>358</v>
       </c>
-      <c r="G8" s="7" t="s">
+      <c r="G8" s="14" t="s">
         <v>123</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="7" t="s">
+      <c r="A9" s="14" t="s">
         <v>361</v>
       </c>
-      <c r="B9" s="7" t="s">
+      <c r="B9" s="14" t="s">
         <v>362</v>
       </c>
-      <c r="C9" s="7">
+      <c r="C9" s="14">
         <v>500</v>
       </c>
-      <c r="D9" s="7">
+      <c r="D9" s="14">
         <v>250</v>
       </c>
-      <c r="E9" s="7" t="s">
+      <c r="E9" s="14" t="s">
         <v>357</v>
       </c>
-      <c r="F9" s="7" t="s">
+      <c r="F9" s="14" t="s">
         <v>358</v>
       </c>
-      <c r="G9" s="7"/>
+      <c r="G9" s="14"/>
     </row>
     <row r="10" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="7" t="s">
+      <c r="A10" s="14" t="s">
         <v>363</v>
       </c>
-      <c r="B10" s="7" t="s">
+      <c r="B10" s="14" t="s">
         <v>364</v>
       </c>
-      <c r="C10" s="7">
+      <c r="C10" s="14">
         <v>750</v>
       </c>
-      <c r="D10" s="7" t="s">
+      <c r="D10" s="14" t="s">
         <v>365</v>
       </c>
-      <c r="E10" s="7" t="s">
+      <c r="E10" s="14" t="s">
         <v>357</v>
       </c>
-      <c r="F10" s="7" t="s">
+      <c r="F10" s="14" t="s">
         <v>366</v>
       </c>
-      <c r="G10" s="7"/>
+      <c r="G10" s="14"/>
     </row>
     <row r="13" spans="1:7" ht="17" x14ac:dyDescent="0.2">
-      <c r="A13" s="10" t="s">
+      <c r="A13" s="20" t="s">
         <v>367</v>
       </c>
     </row>
     <row r="15" spans="1:7" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="1" t="s">
+      <c r="A15" s="13" t="s">
         <v>368</v>
       </c>
-      <c r="B15" s="1" t="s">
+      <c r="B15" s="13" t="s">
         <v>369</v>
       </c>
-      <c r="C15" s="1" t="s">
+      <c r="C15" s="13" t="s">
         <v>100</v>
       </c>
-      <c r="D15" s="1" t="s">
+      <c r="D15" s="13" t="s">
         <v>370</v>
       </c>
-      <c r="E15" s="1" t="s">
+      <c r="E15" s="13" t="s">
         <v>371</v>
       </c>
     </row>
     <row r="16" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="7" t="s">
+      <c r="A16" s="14" t="s">
         <v>372</v>
       </c>
-      <c r="B16" s="7" t="s">
+      <c r="B16" s="14" t="s">
         <v>373</v>
       </c>
-      <c r="C16" s="7" t="s">
+      <c r="C16" s="14" t="s">
         <v>374</v>
       </c>
-      <c r="D16" s="7" t="s">
+      <c r="D16" s="14" t="s">
         <v>375</v>
       </c>
-      <c r="E16" s="7" t="s">
+      <c r="E16" s="14" t="s">
         <v>376</v>
       </c>
     </row>
     <row r="17" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="7" t="s">
+      <c r="A17" s="14" t="s">
         <v>377</v>
       </c>
-      <c r="B17" s="7" t="s">
+      <c r="B17" s="14" t="s">
         <v>355</v>
       </c>
-      <c r="C17" s="7" t="s">
+      <c r="C17" s="14" t="s">
         <v>378</v>
       </c>
-      <c r="D17" s="7" t="s">
+      <c r="D17" s="14" t="s">
         <v>375</v>
       </c>
-      <c r="E17" s="7" t="s">
+      <c r="E17" s="14" t="s">
         <v>379</v>
       </c>
     </row>
     <row r="18" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="7" t="s">
+      <c r="A18" s="14" t="s">
         <v>380</v>
       </c>
-      <c r="B18" s="7" t="s">
+      <c r="B18" s="14" t="s">
         <v>359</v>
       </c>
-      <c r="C18" s="7" t="s">
+      <c r="C18" s="14" t="s">
         <v>378</v>
       </c>
-      <c r="D18" s="7" t="s">
+      <c r="D18" s="14" t="s">
         <v>375</v>
       </c>
-      <c r="E18" s="7" t="s">
+      <c r="E18" s="14" t="s">
         <v>379</v>
       </c>
     </row>
     <row r="19" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="7" t="s">
+      <c r="A19" s="14" t="s">
         <v>381</v>
       </c>
-      <c r="B19" s="7" t="s">
+      <c r="B19" s="14" t="s">
         <v>361</v>
       </c>
-      <c r="C19" s="7" t="s">
+      <c r="C19" s="14" t="s">
         <v>378</v>
       </c>
-      <c r="D19" s="7" t="s">
+      <c r="D19" s="14" t="s">
         <v>375</v>
       </c>
-      <c r="E19" s="7" t="s">
+      <c r="E19" s="14" t="s">
         <v>379</v>
       </c>
     </row>
     <row r="20" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="7" t="s">
+      <c r="A20" s="14" t="s">
         <v>382</v>
       </c>
-      <c r="B20" s="7" t="s">
+      <c r="B20" s="14" t="s">
         <v>363</v>
       </c>
-      <c r="C20" s="7" t="s">
+      <c r="C20" s="14" t="s">
         <v>378</v>
       </c>
-      <c r="D20" s="7" t="s">
+      <c r="D20" s="14" t="s">
         <v>375</v>
       </c>
-      <c r="E20" s="7" t="s">
+      <c r="E20" s="14" t="s">
         <v>379</v>
       </c>
     </row>
     <row r="21" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="7" t="s">
+      <c r="A21" s="14" t="s">
         <v>383</v>
       </c>
-      <c r="B21" s="7" t="s">
+      <c r="B21" s="14" t="s">
         <v>384</v>
       </c>
-      <c r="C21" s="7" t="s">
+      <c r="C21" s="14" t="s">
         <v>385</v>
       </c>
-      <c r="D21" s="7" t="s">
+      <c r="D21" s="14" t="s">
         <v>386</v>
       </c>
-      <c r="E21" s="7" t="s">
+      <c r="E21" s="14" t="s">
         <v>387</v>
       </c>
     </row>
     <row r="22" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="7" t="s">
+      <c r="A22" s="14" t="s">
         <v>388</v>
       </c>
-      <c r="B22" s="7" t="s">
+      <c r="B22" s="14" t="s">
         <v>389</v>
       </c>
-      <c r="C22" s="7" t="s">
+      <c r="C22" s="14" t="s">
         <v>385</v>
       </c>
-      <c r="D22" s="7" t="s">
+      <c r="D22" s="14" t="s">
         <v>386</v>
       </c>
-      <c r="E22" s="7" t="s">
+      <c r="E22" s="14" t="s">
         <v>387</v>
       </c>
     </row>
     <row r="23" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="7" t="s">
+      <c r="A23" s="14" t="s">
         <v>390</v>
       </c>
-      <c r="B23" s="7" t="s">
+      <c r="B23" s="14" t="s">
         <v>391</v>
       </c>
-      <c r="C23" s="7" t="s">
+      <c r="C23" s="14" t="s">
         <v>385</v>
       </c>
-      <c r="D23" s="7" t="s">
+      <c r="D23" s="14" t="s">
         <v>386</v>
       </c>
-      <c r="E23" s="7" t="s">
+      <c r="E23" s="14" t="s">
         <v>387</v>
       </c>
     </row>
@@ -2506,107 +2536,107 @@
   <dimension ref="A1:F9"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="18" style="4" customWidth="1"/>
-    <col min="2" max="2" width="12" style="4" customWidth="1"/>
-    <col min="3" max="5" width="14" style="4" customWidth="1"/>
-    <col min="6" max="16384" width="8.83203125" style="4"/>
+    <col min="1" max="1" width="18" style="15" customWidth="1"/>
+    <col min="2" max="2" width="12" style="15" customWidth="1"/>
+    <col min="3" max="5" width="14" style="15" customWidth="1"/>
+    <col min="6" max="16384" width="8.83203125" style="2"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="21" x14ac:dyDescent="0.2">
-      <c r="A1" s="8" t="s">
+      <c r="A1" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="B1" s="3"/>
-      <c r="C1" s="3"/>
-      <c r="D1" s="3"/>
-      <c r="E1" s="3"/>
-      <c r="F1" s="3"/>
+      <c r="B1" s="6"/>
+      <c r="C1" s="6"/>
+      <c r="D1" s="6"/>
+      <c r="E1" s="6"/>
+      <c r="F1" s="6"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" s="5" t="s">
         <v>392</v>
       </c>
-      <c r="B2" s="3"/>
-      <c r="C2" s="3"/>
-      <c r="D2" s="3"/>
-      <c r="E2" s="3"/>
-      <c r="F2" s="3"/>
+      <c r="B2" s="6"/>
+      <c r="C2" s="6"/>
+      <c r="D2" s="6"/>
+      <c r="E2" s="6"/>
+      <c r="F2" s="6"/>
     </row>
     <row r="4" spans="1:6" ht="45" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="9" t="s">
+      <c r="A4" s="8" t="s">
         <v>393</v>
       </c>
-      <c r="B4" s="3"/>
-      <c r="C4" s="3"/>
-      <c r="D4" s="3"/>
-      <c r="E4" s="3"/>
-      <c r="F4" s="3"/>
+      <c r="B4" s="6"/>
+      <c r="C4" s="6"/>
+      <c r="D4" s="6"/>
+      <c r="E4" s="6"/>
+      <c r="F4" s="6"/>
     </row>
     <row r="6" spans="1:6" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="1" t="s">
+      <c r="A6" s="13" t="s">
         <v>394</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="B6" s="13" t="s">
         <v>263</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="C6" s="13" t="s">
         <v>167</v>
       </c>
-      <c r="D6" s="1" t="s">
+      <c r="D6" s="13" t="s">
         <v>395</v>
       </c>
-      <c r="E6" s="1" t="s">
+      <c r="E6" s="13" t="s">
         <v>396</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="7" t="s">
+      <c r="A7" s="14" t="s">
         <v>397</v>
       </c>
-      <c r="B7" s="7" t="s">
+      <c r="B7" s="14" t="s">
         <v>398</v>
       </c>
-      <c r="C7" s="7" t="s">
+      <c r="C7" s="14" t="s">
         <v>399</v>
       </c>
-      <c r="D7" s="7">
+      <c r="D7" s="14">
         <v>0</v>
       </c>
-      <c r="E7" s="7" t="s">
+      <c r="E7" s="14" t="s">
         <v>90</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="7" t="s">
+      <c r="A8" s="14" t="s">
         <v>400</v>
       </c>
-      <c r="B8" s="7" t="s">
+      <c r="B8" s="14" t="s">
         <v>401</v>
       </c>
-      <c r="C8" s="7" t="s">
+      <c r="C8" s="14" t="s">
         <v>402</v>
       </c>
-      <c r="D8" s="7">
+      <c r="D8" s="14">
         <v>500</v>
       </c>
-      <c r="E8" s="7" t="s">
+      <c r="E8" s="14" t="s">
         <v>403</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="7" t="s">
+      <c r="A9" s="14" t="s">
         <v>404</v>
       </c>
-      <c r="B9" s="7" t="s">
+      <c r="B9" s="14" t="s">
         <v>398</v>
       </c>
-      <c r="C9" s="7" t="s">
+      <c r="C9" s="14" t="s">
         <v>405</v>
       </c>
-      <c r="D9" s="7">
+      <c r="D9" s="14">
         <v>0</v>
       </c>
-      <c r="E9" s="7" t="s">
+      <c r="E9" s="14" t="s">
         <v>90</v>
       </c>
     </row>
@@ -2628,160 +2658,160 @@
   <dimension ref="A1:I9"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="22" style="4" customWidth="1"/>
-    <col min="2" max="2" width="12" style="4" customWidth="1"/>
-    <col min="3" max="3" width="14" style="4" customWidth="1"/>
-    <col min="4" max="4" width="12" style="4" customWidth="1"/>
-    <col min="5" max="5" width="14" style="4" customWidth="1"/>
-    <col min="6" max="6" width="30" style="4" customWidth="1"/>
-    <col min="7" max="7" width="20" style="4" customWidth="1"/>
-    <col min="8" max="9" width="14" style="4" customWidth="1"/>
-    <col min="10" max="16384" width="8.83203125" style="4"/>
+    <col min="1" max="1" width="22" style="15" customWidth="1"/>
+    <col min="2" max="2" width="12" style="15" customWidth="1"/>
+    <col min="3" max="3" width="14" style="15" customWidth="1"/>
+    <col min="4" max="4" width="12" style="15" customWidth="1"/>
+    <col min="5" max="5" width="14" style="15" customWidth="1"/>
+    <col min="6" max="6" width="30" style="15" customWidth="1"/>
+    <col min="7" max="7" width="20" style="15" customWidth="1"/>
+    <col min="8" max="9" width="14" style="15" customWidth="1"/>
+    <col min="10" max="16384" width="8.83203125" style="2"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="21" x14ac:dyDescent="0.2">
-      <c r="A1" s="8" t="s">
+      <c r="A1" s="16" t="s">
         <v>26</v>
       </c>
-      <c r="B1" s="3"/>
-      <c r="C1" s="3"/>
-      <c r="D1" s="3"/>
-      <c r="E1" s="3"/>
-      <c r="F1" s="3"/>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="17"/>
+      <c r="F1" s="17"/>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A2" s="5" t="s">
+      <c r="A2" s="18" t="s">
         <v>406</v>
       </c>
-      <c r="B2" s="3"/>
-      <c r="C2" s="3"/>
-      <c r="D2" s="3"/>
-      <c r="E2" s="3"/>
-      <c r="F2" s="3"/>
+      <c r="B2" s="17"/>
+      <c r="C2" s="17"/>
+      <c r="D2" s="17"/>
+      <c r="E2" s="17"/>
+      <c r="F2" s="17"/>
     </row>
     <row r="4" spans="1:9" ht="45" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="9" t="s">
+      <c r="A4" s="19" t="s">
         <v>407</v>
       </c>
-      <c r="B4" s="3"/>
-      <c r="C4" s="3"/>
-      <c r="D4" s="3"/>
-      <c r="E4" s="3"/>
-      <c r="F4" s="3"/>
+      <c r="B4" s="17"/>
+      <c r="C4" s="17"/>
+      <c r="D4" s="17"/>
+      <c r="E4" s="17"/>
+      <c r="F4" s="17"/>
     </row>
     <row r="6" spans="1:9" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="1" t="s">
+      <c r="A6" s="13" t="s">
         <v>408</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="B6" s="13" t="s">
         <v>395</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="C6" s="13" t="s">
         <v>409</v>
       </c>
-      <c r="D6" s="1" t="s">
+      <c r="D6" s="13" t="s">
         <v>410</v>
       </c>
-      <c r="E6" s="1" t="s">
+      <c r="E6" s="13" t="s">
         <v>411</v>
       </c>
-      <c r="F6" s="1" t="s">
+      <c r="F6" s="13" t="s">
         <v>412</v>
       </c>
-      <c r="G6" s="1" t="s">
+      <c r="G6" s="13" t="s">
         <v>413</v>
       </c>
-      <c r="H6" s="1" t="s">
+      <c r="H6" s="13" t="s">
         <v>414</v>
       </c>
-      <c r="I6" s="1" t="s">
+      <c r="I6" s="13" t="s">
         <v>415</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="7" t="s">
+      <c r="A7" s="14" t="s">
         <v>416</v>
       </c>
-      <c r="B7" s="7">
+      <c r="B7" s="14">
         <v>3200</v>
       </c>
-      <c r="C7" s="7">
+      <c r="C7" s="14">
         <v>500</v>
       </c>
-      <c r="D7" s="7">
+      <c r="D7" s="14">
         <v>12</v>
       </c>
-      <c r="E7" s="7">
+      <c r="E7" s="14">
         <v>225</v>
       </c>
-      <c r="F7" s="7" t="s">
+      <c r="F7" s="14" t="s">
         <v>417</v>
       </c>
-      <c r="G7" s="7" t="s">
+      <c r="G7" s="14" t="s">
         <v>418</v>
       </c>
-      <c r="H7" s="7" t="s">
+      <c r="H7" s="14" t="s">
         <v>419</v>
       </c>
-      <c r="I7" s="7">
+      <c r="I7" s="14">
         <v>300</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="7" t="s">
+      <c r="A8" s="14" t="s">
         <v>420</v>
       </c>
-      <c r="B8" s="7">
+      <c r="B8" s="14">
         <v>3800</v>
       </c>
-      <c r="C8" s="7">
+      <c r="C8" s="14">
         <v>800</v>
       </c>
-      <c r="D8" s="7">
+      <c r="D8" s="14">
         <v>24</v>
       </c>
-      <c r="E8" s="7">
+      <c r="E8" s="14">
         <v>125</v>
       </c>
-      <c r="F8" s="7" t="s">
+      <c r="F8" s="14" t="s">
         <v>421</v>
       </c>
-      <c r="G8" s="7" t="s">
+      <c r="G8" s="14" t="s">
         <v>422</v>
       </c>
-      <c r="H8" s="7" t="s">
+      <c r="H8" s="14" t="s">
         <v>423</v>
       </c>
-      <c r="I8" s="7" t="s">
+      <c r="I8" s="14" t="s">
         <v>90</v>
       </c>
     </row>
     <row r="9" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="7" t="s">
+      <c r="A9" s="14" t="s">
         <v>424</v>
       </c>
-      <c r="B9" s="7">
+      <c r="B9" s="14">
         <v>1200</v>
       </c>
-      <c r="C9" s="7">
+      <c r="C9" s="14">
         <v>200</v>
       </c>
-      <c r="D9" s="7">
+      <c r="D9" s="14">
         <v>6</v>
       </c>
-      <c r="E9" s="7">
+      <c r="E9" s="14">
         <v>167</v>
       </c>
-      <c r="F9" s="7" t="s">
+      <c r="F9" s="14" t="s">
         <v>425</v>
       </c>
-      <c r="G9" s="7" t="s">
+      <c r="G9" s="14" t="s">
         <v>426</v>
       </c>
-      <c r="H9" s="7" t="s">
+      <c r="H9" s="14" t="s">
         <v>419</v>
       </c>
-      <c r="I9" s="7" t="s">
+      <c r="I9" s="14" t="s">
         <v>90</v>
       </c>
     </row>
@@ -2803,201 +2833,201 @@
   <dimension ref="A1:F13"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="14" style="4" customWidth="1"/>
-    <col min="2" max="2" width="16" style="4" customWidth="1"/>
-    <col min="3" max="3" width="22" style="4" customWidth="1"/>
-    <col min="4" max="5" width="16" style="4" customWidth="1"/>
-    <col min="6" max="6" width="70" style="4" customWidth="1"/>
-    <col min="7" max="16384" width="8.83203125" style="4"/>
+    <col min="1" max="1" width="14" style="15" customWidth="1"/>
+    <col min="2" max="2" width="16" style="15" customWidth="1"/>
+    <col min="3" max="3" width="22" style="15" customWidth="1"/>
+    <col min="4" max="5" width="16" style="15" customWidth="1"/>
+    <col min="6" max="6" width="70" style="15" customWidth="1"/>
+    <col min="7" max="16384" width="8.83203125" style="2"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="21" x14ac:dyDescent="0.2">
-      <c r="A1" s="8" t="s">
+      <c r="A1" s="16" t="s">
         <v>28</v>
       </c>
-      <c r="B1" s="3"/>
-      <c r="C1" s="3"/>
-      <c r="D1" s="3"/>
-      <c r="E1" s="3"/>
-      <c r="F1" s="3"/>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="17"/>
+      <c r="F1" s="17"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A2" s="5" t="s">
+      <c r="A2" s="18" t="s">
         <v>427</v>
       </c>
-      <c r="B2" s="3"/>
-      <c r="C2" s="3"/>
-      <c r="D2" s="3"/>
-      <c r="E2" s="3"/>
-      <c r="F2" s="3"/>
+      <c r="B2" s="17"/>
+      <c r="C2" s="17"/>
+      <c r="D2" s="17"/>
+      <c r="E2" s="17"/>
+      <c r="F2" s="17"/>
     </row>
     <row r="4" spans="1:6" ht="45" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="9" t="s">
+      <c r="A4" s="19" t="s">
         <v>428</v>
       </c>
-      <c r="B4" s="3"/>
-      <c r="C4" s="3"/>
-      <c r="D4" s="3"/>
-      <c r="E4" s="3"/>
-      <c r="F4" s="3"/>
+      <c r="B4" s="17"/>
+      <c r="C4" s="17"/>
+      <c r="D4" s="17"/>
+      <c r="E4" s="17"/>
+      <c r="F4" s="17"/>
     </row>
     <row r="6" spans="1:6" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="1" t="s">
+      <c r="A6" s="13" t="s">
         <v>97</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="B6" s="13" t="s">
         <v>99</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="C6" s="13" t="s">
         <v>429</v>
       </c>
-      <c r="D6" s="1" t="s">
+      <c r="D6" s="13" t="s">
         <v>430</v>
       </c>
-      <c r="E6" s="1" t="s">
+      <c r="E6" s="13" t="s">
         <v>431</v>
       </c>
-      <c r="F6" s="1" t="s">
+      <c r="F6" s="13" t="s">
         <v>432</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="7" t="s">
+      <c r="A7" s="14" t="s">
         <v>130</v>
       </c>
-      <c r="B7" s="7" t="s">
+      <c r="B7" s="14" t="s">
         <v>109</v>
       </c>
-      <c r="C7" s="7" t="s">
+      <c r="C7" s="14" t="s">
         <v>433</v>
       </c>
-      <c r="D7" s="7" t="s">
+      <c r="D7" s="14" t="s">
         <v>434</v>
       </c>
-      <c r="E7" s="7" t="s">
+      <c r="E7" s="14" t="s">
         <v>90</v>
       </c>
-      <c r="F7" s="7" t="s">
+      <c r="F7" s="14" t="s">
         <v>435</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="7" t="s">
+      <c r="A8" s="14" t="s">
         <v>143</v>
       </c>
-      <c r="B8" s="7" t="s">
+      <c r="B8" s="14" t="s">
         <v>145</v>
       </c>
-      <c r="C8" s="7" t="s">
+      <c r="C8" s="14" t="s">
         <v>436</v>
       </c>
-      <c r="D8" s="7">
+      <c r="D8" s="14">
         <v>2</v>
       </c>
-      <c r="E8" s="7">
+      <c r="E8" s="14">
         <v>2</v>
       </c>
-      <c r="F8" s="7" t="s">
+      <c r="F8" s="14" t="s">
         <v>437</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="7" t="s">
+      <c r="A9" s="14" t="s">
         <v>116</v>
       </c>
-      <c r="B9" s="7" t="s">
+      <c r="B9" s="14" t="s">
         <v>118</v>
       </c>
-      <c r="C9" s="7" t="s">
+      <c r="C9" s="14" t="s">
         <v>438</v>
       </c>
-      <c r="D9" s="7">
+      <c r="D9" s="14">
         <v>1</v>
       </c>
-      <c r="E9" s="7">
+      <c r="E9" s="14">
         <v>1</v>
       </c>
-      <c r="F9" s="7" t="s">
+      <c r="F9" s="14" t="s">
         <v>439</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="7" t="s">
+      <c r="A10" s="14" t="s">
         <v>107</v>
       </c>
-      <c r="B10" s="7" t="s">
+      <c r="B10" s="14" t="s">
         <v>109</v>
       </c>
-      <c r="C10" s="7" t="s">
+      <c r="C10" s="14" t="s">
         <v>433</v>
       </c>
-      <c r="D10" s="7">
+      <c r="D10" s="14">
         <v>1</v>
       </c>
-      <c r="E10" s="7">
+      <c r="E10" s="14">
         <v>0</v>
       </c>
-      <c r="F10" s="7" t="s">
+      <c r="F10" s="14" t="s">
         <v>440</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="7" t="s">
+      <c r="A11" s="14" t="s">
         <v>125</v>
       </c>
-      <c r="B11" s="7" t="s">
+      <c r="B11" s="14" t="s">
         <v>109</v>
       </c>
-      <c r="C11" s="7" t="s">
+      <c r="C11" s="14" t="s">
         <v>433</v>
       </c>
-      <c r="D11" s="7">
+      <c r="D11" s="14">
         <v>0</v>
       </c>
-      <c r="E11" s="7">
+      <c r="E11" s="14">
         <v>0</v>
       </c>
-      <c r="F11" s="7" t="s">
+      <c r="F11" s="14" t="s">
         <v>441</v>
       </c>
     </row>
     <row r="12" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="7" t="s">
+      <c r="A12" s="14" t="s">
         <v>150</v>
       </c>
-      <c r="B12" s="7" t="s">
+      <c r="B12" s="14" t="s">
         <v>152</v>
       </c>
-      <c r="C12" s="7" t="s">
+      <c r="C12" s="14" t="s">
         <v>442</v>
       </c>
-      <c r="D12" s="7">
+      <c r="D12" s="14">
         <v>0</v>
       </c>
-      <c r="E12" s="7">
+      <c r="E12" s="14">
         <v>0</v>
       </c>
-      <c r="F12" s="7" t="s">
+      <c r="F12" s="14" t="s">
         <v>443</v>
       </c>
     </row>
     <row r="13" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="7" t="s">
+      <c r="A13" s="14" t="s">
         <v>157</v>
       </c>
-      <c r="B13" s="7" t="s">
+      <c r="B13" s="14" t="s">
         <v>109</v>
       </c>
-      <c r="C13" s="7" t="s">
+      <c r="C13" s="14" t="s">
         <v>433</v>
       </c>
-      <c r="D13" s="7">
+      <c r="D13" s="14">
         <v>0</v>
       </c>
-      <c r="E13" s="7">
+      <c r="E13" s="14">
         <v>0</v>
       </c>
-      <c r="F13" s="7" t="s">
+      <c r="F13" s="14" t="s">
         <v>444</v>
       </c>
     </row>
@@ -3019,102 +3049,102 @@
   <dimension ref="A1:F13"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="30" style="4" customWidth="1"/>
-    <col min="2" max="2" width="90" style="4" customWidth="1"/>
-    <col min="3" max="16384" width="8.83203125" style="4"/>
+    <col min="1" max="1" width="30" style="15" customWidth="1"/>
+    <col min="2" max="2" width="90" style="15" customWidth="1"/>
+    <col min="3" max="16384" width="8.83203125" style="2"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="21" x14ac:dyDescent="0.2">
-      <c r="A1" s="8" t="s">
+      <c r="A1" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="B1" s="3"/>
-      <c r="C1" s="3"/>
-      <c r="D1" s="3"/>
-      <c r="E1" s="3"/>
-      <c r="F1" s="3"/>
+      <c r="B1" s="6"/>
+      <c r="C1" s="6"/>
+      <c r="D1" s="6"/>
+      <c r="E1" s="6"/>
+      <c r="F1" s="6"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" s="5" t="s">
         <v>445</v>
       </c>
-      <c r="B2" s="3"/>
-      <c r="C2" s="3"/>
-      <c r="D2" s="3"/>
-      <c r="E2" s="3"/>
-      <c r="F2" s="3"/>
+      <c r="B2" s="6"/>
+      <c r="C2" s="6"/>
+      <c r="D2" s="6"/>
+      <c r="E2" s="6"/>
+      <c r="F2" s="6"/>
     </row>
     <row r="4" spans="1:6" ht="45" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="9" t="s">
+      <c r="A4" s="8" t="s">
         <v>446</v>
       </c>
-      <c r="B4" s="3"/>
-      <c r="C4" s="3"/>
-      <c r="D4" s="3"/>
-      <c r="E4" s="3"/>
-      <c r="F4" s="3"/>
+      <c r="B4" s="6"/>
+      <c r="C4" s="6"/>
+      <c r="D4" s="6"/>
+      <c r="E4" s="6"/>
+      <c r="F4" s="6"/>
     </row>
     <row r="6" spans="1:6" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="1" t="s">
+      <c r="A6" s="13" t="s">
         <v>447</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="B6" s="13" t="s">
         <v>448</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="7" t="s">
+      <c r="A7" s="14" t="s">
         <v>449</v>
       </c>
-      <c r="B7" s="7" t="s">
+      <c r="B7" s="14" t="s">
         <v>450</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="7" t="s">
+      <c r="A8" s="14" t="s">
         <v>451</v>
       </c>
-      <c r="B8" s="7" t="s">
+      <c r="B8" s="14" t="s">
         <v>452</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="7" t="s">
+      <c r="A9" s="14" t="s">
         <v>453</v>
       </c>
-      <c r="B9" s="7" t="s">
+      <c r="B9" s="14" t="s">
         <v>454</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="7" t="s">
+      <c r="A10" s="14" t="s">
         <v>455</v>
       </c>
-      <c r="B10" s="7" t="s">
+      <c r="B10" s="14" t="s">
         <v>456</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="7" t="s">
+      <c r="A11" s="14" t="s">
         <v>457</v>
       </c>
-      <c r="B11" s="7" t="s">
+      <c r="B11" s="14" t="s">
         <v>458</v>
       </c>
     </row>
     <row r="12" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="7" t="s">
+      <c r="A12" s="14" t="s">
         <v>459</v>
       </c>
-      <c r="B12" s="7" t="s">
+      <c r="B12" s="14" t="s">
         <v>460</v>
       </c>
     </row>
     <row r="13" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="7" t="s">
+      <c r="A13" s="14" t="s">
         <v>461</v>
       </c>
-      <c r="B13" s="7" t="s">
+      <c r="B13" s="14" t="s">
         <v>462</v>
       </c>
     </row>
@@ -3136,105 +3166,105 @@
   <dimension ref="A1:F11"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="42" style="4" customWidth="1"/>
-    <col min="2" max="2" width="40" style="4" customWidth="1"/>
-    <col min="3" max="3" width="55" style="4" customWidth="1"/>
-    <col min="4" max="16384" width="8.83203125" style="4"/>
+    <col min="1" max="1" width="42" style="15" customWidth="1"/>
+    <col min="2" max="2" width="40" style="15" customWidth="1"/>
+    <col min="3" max="3" width="55" style="15" customWidth="1"/>
+    <col min="4" max="16384" width="8.83203125" style="2"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="21" x14ac:dyDescent="0.2">
-      <c r="A1" s="8" t="s">
+      <c r="A1" s="7" t="s">
         <v>463</v>
       </c>
-      <c r="B1" s="3"/>
-      <c r="C1" s="3"/>
-      <c r="D1" s="3"/>
-      <c r="E1" s="3"/>
-      <c r="F1" s="3"/>
+      <c r="B1" s="6"/>
+      <c r="C1" s="6"/>
+      <c r="D1" s="6"/>
+      <c r="E1" s="6"/>
+      <c r="F1" s="6"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" s="5" t="s">
         <v>464</v>
       </c>
-      <c r="B2" s="3"/>
-      <c r="C2" s="3"/>
-      <c r="D2" s="3"/>
-      <c r="E2" s="3"/>
-      <c r="F2" s="3"/>
+      <c r="B2" s="6"/>
+      <c r="C2" s="6"/>
+      <c r="D2" s="6"/>
+      <c r="E2" s="6"/>
+      <c r="F2" s="6"/>
     </row>
     <row r="4" spans="1:6" ht="45" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="9" t="s">
+      <c r="A4" s="8" t="s">
         <v>465</v>
       </c>
-      <c r="B4" s="3"/>
-      <c r="C4" s="3"/>
-      <c r="D4" s="3"/>
-      <c r="E4" s="3"/>
-      <c r="F4" s="3"/>
+      <c r="B4" s="6"/>
+      <c r="C4" s="6"/>
+      <c r="D4" s="6"/>
+      <c r="E4" s="6"/>
+      <c r="F4" s="6"/>
     </row>
     <row r="6" spans="1:6" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="1" t="s">
+      <c r="A6" s="13" t="s">
         <v>466</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="B6" s="13" t="s">
         <v>467</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="C6" s="13" t="s">
         <v>106</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="7" t="s">
+      <c r="A7" s="14" t="s">
         <v>468</v>
       </c>
-      <c r="B7" s="7" t="s">
+      <c r="B7" s="14" t="s">
         <v>47</v>
       </c>
-      <c r="C7" s="7" t="s">
+      <c r="C7" s="14" t="s">
         <v>469</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="7" t="s">
+      <c r="A8" s="14" t="s">
         <v>470</v>
       </c>
-      <c r="B8" s="7" t="s">
+      <c r="B8" s="14" t="s">
         <v>471</v>
       </c>
-      <c r="C8" s="7" t="s">
+      <c r="C8" s="14" t="s">
         <v>472</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="7" t="s">
+      <c r="A9" s="14" t="s">
         <v>473</v>
       </c>
-      <c r="B9" s="7" t="s">
+      <c r="B9" s="14" t="s">
         <v>471</v>
       </c>
-      <c r="C9" s="7" t="s">
+      <c r="C9" s="14" t="s">
         <v>474</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="7" t="s">
+      <c r="A10" s="14" t="s">
         <v>475</v>
       </c>
-      <c r="B10" s="7" t="s">
+      <c r="B10" s="14" t="s">
         <v>471</v>
       </c>
-      <c r="C10" s="7" t="s">
+      <c r="C10" s="14" t="s">
         <v>476</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="7" t="s">
+      <c r="A11" s="14" t="s">
         <v>477</v>
       </c>
-      <c r="B11" s="7" t="s">
+      <c r="B11" s="14" t="s">
         <v>478</v>
       </c>
-      <c r="C11" s="7" t="s">
+      <c r="C11" s="14" t="s">
         <v>479</v>
       </c>
     </row>
@@ -3256,366 +3286,366 @@
   <dimension ref="A1:J15"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="16" style="4" customWidth="1"/>
-    <col min="2" max="2" width="14" style="4" customWidth="1"/>
-    <col min="3" max="3" width="26" style="4" customWidth="1"/>
-    <col min="4" max="4" width="22" style="4" customWidth="1"/>
-    <col min="5" max="5" width="20" style="4" customWidth="1"/>
-    <col min="6" max="6" width="18" style="4" customWidth="1"/>
-    <col min="7" max="7" width="24" style="4" customWidth="1"/>
-    <col min="8" max="8" width="18" style="4" customWidth="1"/>
-    <col min="9" max="9" width="16" style="4" customWidth="1"/>
-    <col min="10" max="10" width="60" style="4" customWidth="1"/>
-    <col min="11" max="16384" width="8.83203125" style="4"/>
+    <col min="1" max="1" width="16" style="15" customWidth="1"/>
+    <col min="2" max="2" width="14" style="15" customWidth="1"/>
+    <col min="3" max="3" width="26" style="15" customWidth="1"/>
+    <col min="4" max="4" width="22" style="15" customWidth="1"/>
+    <col min="5" max="5" width="20" style="15" customWidth="1"/>
+    <col min="6" max="6" width="18" style="15" customWidth="1"/>
+    <col min="7" max="7" width="24" style="15" customWidth="1"/>
+    <col min="8" max="8" width="18" style="15" customWidth="1"/>
+    <col min="9" max="9" width="16" style="15" customWidth="1"/>
+    <col min="10" max="10" width="60" style="15" customWidth="1"/>
+    <col min="11" max="16384" width="8.83203125" style="2"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="21" x14ac:dyDescent="0.2">
-      <c r="A1" s="8" t="s">
+      <c r="A1" s="16" t="s">
         <v>4</v>
       </c>
-      <c r="B1" s="3"/>
-      <c r="C1" s="3"/>
-      <c r="D1" s="3"/>
-      <c r="E1" s="3"/>
-      <c r="F1" s="3"/>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="17"/>
+      <c r="F1" s="17"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A2" s="5" t="s">
+      <c r="A2" s="18" t="s">
         <v>34</v>
       </c>
-      <c r="B2" s="3"/>
-      <c r="C2" s="3"/>
-      <c r="D2" s="3"/>
-      <c r="E2" s="3"/>
-      <c r="F2" s="3"/>
+      <c r="B2" s="17"/>
+      <c r="C2" s="17"/>
+      <c r="D2" s="17"/>
+      <c r="E2" s="17"/>
+      <c r="F2" s="17"/>
     </row>
     <row r="4" spans="1:10" ht="45" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="9" t="s">
+      <c r="A4" s="19" t="s">
         <v>35</v>
       </c>
-      <c r="B4" s="3"/>
-      <c r="C4" s="3"/>
-      <c r="D4" s="3"/>
-      <c r="E4" s="3"/>
-      <c r="F4" s="3"/>
+      <c r="B4" s="17"/>
+      <c r="C4" s="17"/>
+      <c r="D4" s="17"/>
+      <c r="E4" s="17"/>
+      <c r="F4" s="17"/>
     </row>
     <row r="6" spans="1:10" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="1" t="s">
+      <c r="A6" s="13" t="s">
         <v>36</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="B6" s="13" t="s">
         <v>37</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="C6" s="13" t="s">
         <v>38</v>
       </c>
-      <c r="D6" s="1" t="s">
+      <c r="D6" s="13" t="s">
         <v>39</v>
       </c>
-      <c r="E6" s="1" t="s">
+      <c r="E6" s="13" t="s">
         <v>40</v>
       </c>
-      <c r="F6" s="1" t="s">
+      <c r="F6" s="13" t="s">
         <v>41</v>
       </c>
-      <c r="G6" s="1" t="s">
+      <c r="G6" s="13" t="s">
         <v>42</v>
       </c>
-      <c r="H6" s="1" t="s">
+      <c r="H6" s="13" t="s">
         <v>43</v>
       </c>
-      <c r="I6" s="1" t="s">
+      <c r="I6" s="13" t="s">
         <v>44</v>
       </c>
-      <c r="J6" s="1" t="s">
+      <c r="J6" s="13" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="7" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="7" t="s">
+      <c r="A7" s="14" t="s">
         <v>46</v>
       </c>
-      <c r="B7" s="7" t="s">
+      <c r="B7" s="14" t="s">
         <v>47</v>
       </c>
-      <c r="C7" s="7" t="s">
+      <c r="C7" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="D7" s="7" t="s">
+      <c r="D7" s="14" t="s">
         <v>49</v>
       </c>
-      <c r="E7" s="7" t="s">
+      <c r="E7" s="14" t="s">
         <v>50</v>
       </c>
-      <c r="F7" s="7" t="s">
+      <c r="F7" s="14" t="s">
         <v>51</v>
       </c>
-      <c r="G7" s="7" t="s">
+      <c r="G7" s="14" t="s">
         <v>52</v>
       </c>
-      <c r="H7" s="7" t="s">
+      <c r="H7" s="14" t="s">
         <v>53</v>
       </c>
-      <c r="I7" s="7" t="s">
+      <c r="I7" s="14" t="s">
         <v>54</v>
       </c>
-      <c r="J7" s="7" t="s">
+      <c r="J7" s="14" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="8" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="7" t="s">
+      <c r="A8" s="14" t="s">
         <v>56</v>
       </c>
-      <c r="B8" s="7" t="s">
+      <c r="B8" s="14" t="s">
         <v>47</v>
       </c>
-      <c r="C8" s="7" t="s">
+      <c r="C8" s="14" t="s">
         <v>57</v>
       </c>
-      <c r="D8" s="7" t="s">
+      <c r="D8" s="14" t="s">
         <v>49</v>
       </c>
-      <c r="E8" s="7" t="s">
+      <c r="E8" s="14" t="s">
         <v>50</v>
       </c>
-      <c r="F8" s="7" t="s">
+      <c r="F8" s="14" t="s">
         <v>58</v>
       </c>
-      <c r="G8" s="7" t="s">
+      <c r="G8" s="14" t="s">
         <v>59</v>
       </c>
-      <c r="H8" s="7" t="s">
+      <c r="H8" s="14" t="s">
         <v>60</v>
       </c>
-      <c r="I8" s="7" t="s">
+      <c r="I8" s="14" t="s">
         <v>61</v>
       </c>
-      <c r="J8" s="7" t="s">
+      <c r="J8" s="14" t="s">
         <v>62</v>
       </c>
     </row>
     <row r="9" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="7" t="s">
+      <c r="A9" s="14" t="s">
         <v>63</v>
       </c>
-      <c r="B9" s="7" t="s">
+      <c r="B9" s="14" t="s">
         <v>47</v>
       </c>
-      <c r="C9" s="7" t="s">
+      <c r="C9" s="14" t="s">
         <v>64</v>
       </c>
-      <c r="D9" s="7" t="s">
+      <c r="D9" s="14" t="s">
         <v>65</v>
       </c>
-      <c r="E9" s="7" t="s">
+      <c r="E9" s="14" t="s">
         <v>66</v>
       </c>
-      <c r="F9" s="7" t="s">
+      <c r="F9" s="14" t="s">
         <v>67</v>
       </c>
-      <c r="G9" s="7" t="s">
+      <c r="G9" s="14" t="s">
         <v>68</v>
       </c>
-      <c r="H9" s="7" t="s">
+      <c r="H9" s="14" t="s">
         <v>69</v>
       </c>
-      <c r="I9" s="7" t="s">
+      <c r="I9" s="14" t="s">
         <v>70</v>
       </c>
-      <c r="J9" s="7" t="s">
+      <c r="J9" s="14" t="s">
         <v>71</v>
       </c>
     </row>
     <row r="10" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="7" t="s">
+      <c r="A10" s="14" t="s">
         <v>72</v>
       </c>
-      <c r="B10" s="7" t="s">
+      <c r="B10" s="14" t="s">
         <v>47</v>
       </c>
-      <c r="C10" s="7" t="s">
+      <c r="C10" s="14" t="s">
         <v>73</v>
       </c>
-      <c r="D10" s="7" t="s">
+      <c r="D10" s="14" t="s">
         <v>65</v>
       </c>
-      <c r="E10" s="7" t="s">
+      <c r="E10" s="14" t="s">
         <v>66</v>
       </c>
-      <c r="F10" s="7" t="s">
+      <c r="F10" s="14" t="s">
         <v>58</v>
       </c>
-      <c r="G10" s="7" t="s">
+      <c r="G10" s="14" t="s">
         <v>59</v>
       </c>
-      <c r="H10" s="7" t="s">
+      <c r="H10" s="14" t="s">
         <v>60</v>
       </c>
-      <c r="I10" s="7" t="s">
+      <c r="I10" s="14" t="s">
         <v>61</v>
       </c>
-      <c r="J10" s="7" t="s">
+      <c r="J10" s="14" t="s">
         <v>74</v>
       </c>
     </row>
     <row r="11" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="7" t="s">
+      <c r="A11" s="14" t="s">
         <v>75</v>
       </c>
-      <c r="B11" s="7" t="s">
+      <c r="B11" s="14" t="s">
         <v>47</v>
       </c>
-      <c r="C11" s="7" t="s">
+      <c r="C11" s="14" t="s">
         <v>76</v>
       </c>
-      <c r="D11" s="7" t="s">
+      <c r="D11" s="14" t="s">
         <v>77</v>
       </c>
-      <c r="E11" s="7" t="s">
+      <c r="E11" s="14" t="s">
         <v>66</v>
       </c>
-      <c r="F11" s="7" t="s">
+      <c r="F11" s="14" t="s">
         <v>58</v>
       </c>
-      <c r="G11" s="7" t="s">
+      <c r="G11" s="14" t="s">
         <v>59</v>
       </c>
-      <c r="H11" s="7" t="s">
+      <c r="H11" s="14" t="s">
         <v>60</v>
       </c>
-      <c r="I11" s="7" t="s">
+      <c r="I11" s="14" t="s">
         <v>61</v>
       </c>
-      <c r="J11" s="7" t="s">
+      <c r="J11" s="14" t="s">
         <v>78</v>
       </c>
     </row>
     <row r="12" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="7" t="s">
+      <c r="A12" s="14" t="s">
         <v>79</v>
       </c>
-      <c r="B12" s="7" t="s">
+      <c r="B12" s="14" t="s">
         <v>47</v>
       </c>
-      <c r="C12" s="7" t="s">
+      <c r="C12" s="14" t="s">
         <v>80</v>
       </c>
-      <c r="D12" s="7" t="s">
+      <c r="D12" s="14" t="s">
         <v>81</v>
       </c>
-      <c r="E12" s="7" t="s">
+      <c r="E12" s="14" t="s">
         <v>82</v>
       </c>
-      <c r="F12" s="7" t="s">
+      <c r="F12" s="14" t="s">
         <v>51</v>
       </c>
-      <c r="G12" s="7" t="s">
+      <c r="G12" s="14" t="s">
         <v>52</v>
       </c>
-      <c r="H12" s="7" t="s">
+      <c r="H12" s="14" t="s">
         <v>53</v>
       </c>
-      <c r="I12" s="7" t="s">
+      <c r="I12" s="14" t="s">
         <v>54</v>
       </c>
-      <c r="J12" s="7" t="s">
+      <c r="J12" s="14" t="s">
         <v>83</v>
       </c>
     </row>
     <row r="13" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="7" t="s">
+      <c r="A13" s="14" t="s">
         <v>84</v>
       </c>
-      <c r="B13" s="7" t="s">
+      <c r="B13" s="14" t="s">
         <v>47</v>
       </c>
-      <c r="C13" s="7" t="s">
+      <c r="C13" s="14" t="s">
         <v>85</v>
       </c>
-      <c r="D13" s="7" t="s">
+      <c r="D13" s="14" t="s">
         <v>86</v>
       </c>
-      <c r="E13" s="7" t="s">
+      <c r="E13" s="14" t="s">
         <v>82</v>
       </c>
-      <c r="F13" s="7" t="s">
+      <c r="F13" s="14" t="s">
         <v>51</v>
       </c>
-      <c r="G13" s="7" t="s">
+      <c r="G13" s="14" t="s">
         <v>52</v>
       </c>
-      <c r="H13" s="7" t="s">
+      <c r="H13" s="14" t="s">
         <v>53</v>
       </c>
-      <c r="I13" s="7" t="s">
+      <c r="I13" s="14" t="s">
         <v>54</v>
       </c>
-      <c r="J13" s="7" t="s">
+      <c r="J13" s="14" t="s">
         <v>87</v>
       </c>
     </row>
     <row r="14" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="7" t="s">
+      <c r="A14" s="14" t="s">
         <v>88</v>
       </c>
-      <c r="B14" s="7" t="s">
+      <c r="B14" s="14" t="s">
         <v>89</v>
       </c>
-      <c r="C14" s="7" t="s">
+      <c r="C14" s="14" t="s">
         <v>90</v>
       </c>
-      <c r="D14" s="7" t="s">
+      <c r="D14" s="14" t="s">
         <v>90</v>
       </c>
-      <c r="E14" s="7" t="s">
+      <c r="E14" s="14" t="s">
         <v>90</v>
       </c>
-      <c r="F14" s="7" t="s">
+      <c r="F14" s="14" t="s">
         <v>90</v>
       </c>
-      <c r="G14" s="7" t="s">
+      <c r="G14" s="14" t="s">
         <v>90</v>
       </c>
-      <c r="H14" s="7" t="s">
+      <c r="H14" s="14" t="s">
         <v>90</v>
       </c>
-      <c r="I14" s="7" t="s">
+      <c r="I14" s="14" t="s">
         <v>90</v>
       </c>
-      <c r="J14" s="7" t="s">
+      <c r="J14" s="14" t="s">
         <v>91</v>
       </c>
     </row>
     <row r="15" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="7" t="s">
+      <c r="A15" s="14" t="s">
         <v>92</v>
       </c>
-      <c r="B15" s="7" t="s">
+      <c r="B15" s="14" t="s">
         <v>93</v>
       </c>
-      <c r="C15" s="7" t="s">
+      <c r="C15" s="14" t="s">
         <v>90</v>
       </c>
-      <c r="D15" s="7" t="s">
+      <c r="D15" s="14" t="s">
         <v>90</v>
       </c>
-      <c r="E15" s="7" t="s">
+      <c r="E15" s="14" t="s">
         <v>90</v>
       </c>
-      <c r="F15" s="7" t="s">
+      <c r="F15" s="14" t="s">
         <v>90</v>
       </c>
-      <c r="G15" s="7" t="s">
+      <c r="G15" s="14" t="s">
         <v>90</v>
       </c>
-      <c r="H15" s="7" t="s">
+      <c r="H15" s="14" t="s">
         <v>90</v>
       </c>
-      <c r="I15" s="7" t="s">
+      <c r="I15" s="14" t="s">
         <v>90</v>
       </c>
-      <c r="J15" s="7" t="s">
+      <c r="J15" s="14" t="s">
         <v>94</v>
       </c>
     </row>
@@ -3637,333 +3667,333 @@
   <dimension ref="A1:J14"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="14" style="4" customWidth="1"/>
-    <col min="2" max="2" width="20" style="4" customWidth="1"/>
-    <col min="3" max="3" width="12" style="4" customWidth="1"/>
-    <col min="4" max="4" width="24" style="4" customWidth="1"/>
-    <col min="5" max="5" width="16" style="4" customWidth="1"/>
-    <col min="6" max="6" width="30" style="4" customWidth="1"/>
-    <col min="7" max="7" width="18" style="4" customWidth="1"/>
-    <col min="8" max="9" width="14" style="4" customWidth="1"/>
-    <col min="10" max="10" width="60" style="4" customWidth="1"/>
-    <col min="11" max="16384" width="8.83203125" style="4"/>
+    <col min="1" max="1" width="14" style="15" customWidth="1"/>
+    <col min="2" max="2" width="20" style="15" customWidth="1"/>
+    <col min="3" max="3" width="12" style="10" customWidth="1"/>
+    <col min="4" max="4" width="24" style="15" customWidth="1"/>
+    <col min="5" max="5" width="16" style="15" customWidth="1"/>
+    <col min="6" max="6" width="30" style="15" customWidth="1"/>
+    <col min="7" max="7" width="18" style="15" customWidth="1"/>
+    <col min="8" max="9" width="14" style="10" customWidth="1"/>
+    <col min="10" max="10" width="60" style="15" customWidth="1"/>
+    <col min="11" max="16384" width="8.83203125" style="2"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="21" x14ac:dyDescent="0.2">
-      <c r="A1" s="8" t="s">
+      <c r="A1" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="B1" s="3"/>
-      <c r="C1" s="3"/>
-      <c r="D1" s="3"/>
-      <c r="E1" s="3"/>
-      <c r="F1" s="3"/>
+      <c r="B1" s="6"/>
+      <c r="C1" s="6"/>
+      <c r="D1" s="6"/>
+      <c r="E1" s="6"/>
+      <c r="F1" s="6"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A2" s="5" t="s">
         <v>95</v>
       </c>
-      <c r="B2" s="3"/>
-      <c r="C2" s="3"/>
-      <c r="D2" s="3"/>
-      <c r="E2" s="3"/>
-      <c r="F2" s="3"/>
+      <c r="B2" s="6"/>
+      <c r="C2" s="6"/>
+      <c r="D2" s="6"/>
+      <c r="E2" s="6"/>
+      <c r="F2" s="6"/>
     </row>
     <row r="4" spans="1:10" ht="45" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="9" t="s">
+      <c r="A4" s="8" t="s">
         <v>96</v>
       </c>
-      <c r="B4" s="3"/>
-      <c r="C4" s="3"/>
-      <c r="D4" s="3"/>
-      <c r="E4" s="3"/>
-      <c r="F4" s="3"/>
+      <c r="B4" s="6"/>
+      <c r="C4" s="6"/>
+      <c r="D4" s="6"/>
+      <c r="E4" s="6"/>
+      <c r="F4" s="6"/>
     </row>
     <row r="6" spans="1:10" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="1" t="s">
+      <c r="A6" s="13" t="s">
         <v>97</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="B6" s="13" t="s">
         <v>98</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="C6" s="11" t="s">
         <v>99</v>
       </c>
-      <c r="D6" s="1" t="s">
+      <c r="D6" s="13" t="s">
         <v>100</v>
       </c>
-      <c r="E6" s="1" t="s">
+      <c r="E6" s="13" t="s">
         <v>101</v>
       </c>
-      <c r="F6" s="1" t="s">
+      <c r="F6" s="13" t="s">
         <v>102</v>
       </c>
-      <c r="G6" s="1" t="s">
+      <c r="G6" s="13" t="s">
         <v>103</v>
       </c>
-      <c r="H6" s="1" t="s">
+      <c r="H6" s="11" t="s">
         <v>104</v>
       </c>
-      <c r="I6" s="1" t="s">
+      <c r="I6" s="11" t="s">
         <v>105</v>
       </c>
-      <c r="J6" s="1" t="s">
+      <c r="J6" s="13" t="s">
         <v>106</v>
       </c>
     </row>
     <row r="7" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="7" t="s">
+      <c r="A7" s="14" t="s">
         <v>107</v>
       </c>
-      <c r="B7" s="7" t="s">
+      <c r="B7" s="14" t="s">
         <v>108</v>
       </c>
-      <c r="C7" s="7" t="s">
+      <c r="C7" s="12" t="s">
         <v>109</v>
       </c>
-      <c r="D7" s="7" t="s">
+      <c r="D7" s="14" t="s">
         <v>110</v>
       </c>
-      <c r="E7" s="7" t="s">
+      <c r="E7" s="14" t="s">
         <v>111</v>
       </c>
-      <c r="F7" s="7" t="s">
+      <c r="F7" s="14" t="s">
         <v>112</v>
       </c>
-      <c r="G7" s="7" t="s">
+      <c r="G7" s="14" t="s">
         <v>113</v>
       </c>
-      <c r="H7" s="7" t="s">
+      <c r="H7" s="12" t="s">
         <v>114</v>
       </c>
-      <c r="I7" s="7" t="s">
+      <c r="I7" s="12" t="s">
         <v>114</v>
       </c>
-      <c r="J7" s="7" t="s">
+      <c r="J7" s="14" t="s">
         <v>115</v>
       </c>
     </row>
     <row r="8" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="7" t="s">
+      <c r="A8" s="14" t="s">
         <v>116</v>
       </c>
-      <c r="B8" s="7" t="s">
+      <c r="B8" s="14" t="s">
         <v>117</v>
       </c>
-      <c r="C8" s="7" t="s">
+      <c r="C8" s="12" t="s">
         <v>118</v>
       </c>
-      <c r="D8" s="7" t="s">
+      <c r="D8" s="14" t="s">
         <v>119</v>
       </c>
-      <c r="E8" s="7" t="s">
+      <c r="E8" s="14" t="s">
         <v>120</v>
       </c>
-      <c r="F8" s="7" t="s">
+      <c r="F8" s="14" t="s">
         <v>121</v>
       </c>
-      <c r="G8" s="7" t="s">
+      <c r="G8" s="14" t="s">
         <v>122</v>
       </c>
-      <c r="H8" s="7" t="s">
+      <c r="H8" s="12" t="s">
         <v>114</v>
       </c>
-      <c r="I8" s="7" t="s">
+      <c r="I8" s="12" t="s">
         <v>123</v>
       </c>
-      <c r="J8" s="7" t="s">
+      <c r="J8" s="14" t="s">
         <v>124</v>
       </c>
     </row>
     <row r="9" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="7" t="s">
+      <c r="A9" s="14" t="s">
         <v>125</v>
       </c>
-      <c r="B9" s="7" t="s">
+      <c r="B9" s="14" t="s">
         <v>126</v>
       </c>
-      <c r="C9" s="7" t="s">
+      <c r="C9" s="12" t="s">
         <v>109</v>
       </c>
-      <c r="D9" s="7" t="s">
+      <c r="D9" s="14" t="s">
         <v>51</v>
       </c>
-      <c r="E9" s="7" t="s">
+      <c r="E9" s="14" t="s">
         <v>127</v>
       </c>
-      <c r="F9" s="7" t="s">
+      <c r="F9" s="14" t="s">
         <v>128</v>
       </c>
-      <c r="G9" s="7" t="s">
+      <c r="G9" s="14" t="s">
         <v>113</v>
       </c>
-      <c r="H9" s="7" t="s">
+      <c r="H9" s="12" t="s">
         <v>114</v>
       </c>
-      <c r="I9" s="7" t="s">
+      <c r="I9" s="12" t="s">
         <v>114</v>
       </c>
-      <c r="J9" s="7" t="s">
+      <c r="J9" s="14" t="s">
         <v>129</v>
       </c>
     </row>
     <row r="10" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="7" t="s">
+      <c r="A10" s="14" t="s">
         <v>130</v>
       </c>
-      <c r="B10" s="7" t="s">
+      <c r="B10" s="14" t="s">
         <v>131</v>
       </c>
-      <c r="C10" s="7" t="s">
+      <c r="C10" s="12" t="s">
         <v>109</v>
       </c>
-      <c r="D10" s="7" t="s">
+      <c r="D10" s="14" t="s">
         <v>132</v>
       </c>
-      <c r="E10" s="7" t="s">
+      <c r="E10" s="14" t="s">
         <v>133</v>
       </c>
-      <c r="F10" s="7" t="s">
+      <c r="F10" s="14" t="s">
         <v>134</v>
       </c>
-      <c r="G10" s="7" t="s">
+      <c r="G10" s="14" t="s">
         <v>113</v>
       </c>
-      <c r="H10" s="7" t="s">
+      <c r="H10" s="12" t="s">
         <v>123</v>
       </c>
-      <c r="I10" s="7" t="s">
+      <c r="I10" s="12" t="s">
         <v>114</v>
       </c>
-      <c r="J10" s="7" t="s">
+      <c r="J10" s="14" t="s">
         <v>135</v>
       </c>
     </row>
     <row r="11" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="7" t="s">
+      <c r="A11" s="14" t="s">
         <v>136</v>
       </c>
-      <c r="B11" s="7" t="s">
+      <c r="B11" s="14" t="s">
         <v>137</v>
       </c>
-      <c r="C11" s="7" t="s">
+      <c r="C11" s="12" t="s">
         <v>109</v>
       </c>
-      <c r="D11" s="7" t="s">
+      <c r="D11" s="14" t="s">
         <v>138</v>
       </c>
-      <c r="E11" s="7" t="s">
+      <c r="E11" s="14" t="s">
         <v>139</v>
       </c>
-      <c r="F11" s="7" t="s">
+      <c r="F11" s="14" t="s">
         <v>140</v>
       </c>
-      <c r="G11" s="7" t="s">
+      <c r="G11" s="14" t="s">
         <v>141</v>
       </c>
-      <c r="H11" s="7" t="s">
+      <c r="H11" s="12" t="s">
         <v>114</v>
       </c>
-      <c r="I11" s="7" t="s">
+      <c r="I11" s="12" t="s">
         <v>114</v>
       </c>
-      <c r="J11" s="7" t="s">
+      <c r="J11" s="14" t="s">
         <v>142</v>
       </c>
     </row>
     <row r="12" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="7" t="s">
+      <c r="A12" s="14" t="s">
         <v>143</v>
       </c>
-      <c r="B12" s="7" t="s">
+      <c r="B12" s="14" t="s">
         <v>144</v>
       </c>
-      <c r="C12" s="7" t="s">
+      <c r="C12" s="12" t="s">
         <v>145</v>
       </c>
-      <c r="D12" s="7" t="s">
+      <c r="D12" s="14" t="s">
         <v>146</v>
       </c>
-      <c r="E12" s="7" t="s">
+      <c r="E12" s="14" t="s">
         <v>147</v>
       </c>
-      <c r="F12" s="7" t="s">
+      <c r="F12" s="14" t="s">
         <v>148</v>
       </c>
-      <c r="G12" s="7" t="s">
+      <c r="G12" s="14" t="s">
         <v>113</v>
       </c>
-      <c r="H12" s="7" t="s">
+      <c r="H12" s="12" t="s">
         <v>114</v>
       </c>
-      <c r="I12" s="7" t="s">
+      <c r="I12" s="12" t="s">
         <v>114</v>
       </c>
-      <c r="J12" s="7" t="s">
+      <c r="J12" s="14" t="s">
         <v>149</v>
       </c>
     </row>
     <row r="13" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="7" t="s">
+      <c r="A13" s="14" t="s">
         <v>150</v>
       </c>
-      <c r="B13" s="7" t="s">
+      <c r="B13" s="14" t="s">
         <v>151</v>
       </c>
-      <c r="C13" s="7" t="s">
+      <c r="C13" s="12" t="s">
         <v>152</v>
       </c>
-      <c r="D13" s="7" t="s">
+      <c r="D13" s="14" t="s">
         <v>153</v>
       </c>
-      <c r="E13" s="7" t="s">
+      <c r="E13" s="14" t="s">
         <v>154</v>
       </c>
-      <c r="F13" s="7" t="s">
+      <c r="F13" s="14" t="s">
         <v>155</v>
       </c>
-      <c r="G13" s="7" t="s">
+      <c r="G13" s="14" t="s">
         <v>113</v>
       </c>
-      <c r="H13" s="7" t="s">
+      <c r="H13" s="12" t="s">
         <v>114</v>
       </c>
-      <c r="I13" s="7" t="s">
+      <c r="I13" s="12" t="s">
         <v>114</v>
       </c>
-      <c r="J13" s="7" t="s">
+      <c r="J13" s="14" t="s">
         <v>156</v>
       </c>
     </row>
     <row r="14" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="7" t="s">
+      <c r="A14" s="14" t="s">
         <v>157</v>
       </c>
-      <c r="B14" s="7" t="s">
+      <c r="B14" s="14" t="s">
         <v>158</v>
       </c>
-      <c r="C14" s="7" t="s">
+      <c r="C14" s="12" t="s">
         <v>109</v>
       </c>
-      <c r="D14" s="7" t="s">
+      <c r="D14" s="14" t="s">
         <v>159</v>
       </c>
-      <c r="E14" s="7" t="s">
+      <c r="E14" s="14" t="s">
         <v>160</v>
       </c>
-      <c r="F14" s="7" t="s">
+      <c r="F14" s="14" t="s">
         <v>161</v>
       </c>
-      <c r="G14" s="7" t="s">
+      <c r="G14" s="14" t="s">
         <v>113</v>
       </c>
-      <c r="H14" s="7" t="s">
+      <c r="H14" s="12" t="s">
         <v>114</v>
       </c>
-      <c r="I14" s="7" t="s">
+      <c r="I14" s="12" t="s">
         <v>114</v>
       </c>
-      <c r="J14" s="7" t="s">
+      <c r="J14" s="14" t="s">
         <v>162</v>
       </c>
     </row>
@@ -3974,6 +4004,7 @@
     <mergeCell ref="A4:F4"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="8" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
   <headerFooter>
     <oddFooter>&amp;L_x000D_&amp;1#&amp;"Aptos"&amp;10&amp;K000000 Public</oddFooter>
   </headerFooter>
@@ -3985,161 +4016,161 @@
   <dimension ref="A1:F11"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="2" width="14" style="4" customWidth="1"/>
-    <col min="3" max="3" width="30" style="4" customWidth="1"/>
-    <col min="4" max="4" width="12" style="4" customWidth="1"/>
-    <col min="5" max="5" width="18" style="4" customWidth="1"/>
-    <col min="6" max="6" width="34" style="4" customWidth="1"/>
-    <col min="7" max="16384" width="8.83203125" style="4"/>
+    <col min="1" max="2" width="14" style="15" customWidth="1"/>
+    <col min="3" max="3" width="30" style="15" customWidth="1"/>
+    <col min="4" max="4" width="12" style="15" customWidth="1"/>
+    <col min="5" max="5" width="18" style="15" customWidth="1"/>
+    <col min="6" max="6" width="34" style="15" customWidth="1"/>
+    <col min="7" max="16384" width="8.83203125" style="2"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="21" x14ac:dyDescent="0.2">
-      <c r="A1" s="8" t="s">
+      <c r="A1" s="16" t="s">
         <v>8</v>
       </c>
-      <c r="B1" s="3"/>
-      <c r="C1" s="3"/>
-      <c r="D1" s="3"/>
-      <c r="E1" s="3"/>
-      <c r="F1" s="3"/>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="17"/>
+      <c r="F1" s="17"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A2" s="5" t="s">
+      <c r="A2" s="18" t="s">
         <v>163</v>
       </c>
-      <c r="B2" s="3"/>
-      <c r="C2" s="3"/>
-      <c r="D2" s="3"/>
-      <c r="E2" s="3"/>
-      <c r="F2" s="3"/>
+      <c r="B2" s="17"/>
+      <c r="C2" s="17"/>
+      <c r="D2" s="17"/>
+      <c r="E2" s="17"/>
+      <c r="F2" s="17"/>
     </row>
     <row r="4" spans="1:6" ht="45" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="9" t="s">
+      <c r="A4" s="19" t="s">
         <v>164</v>
       </c>
-      <c r="B4" s="3"/>
-      <c r="C4" s="3"/>
-      <c r="D4" s="3"/>
-      <c r="E4" s="3"/>
-      <c r="F4" s="3"/>
+      <c r="B4" s="17"/>
+      <c r="C4" s="17"/>
+      <c r="D4" s="17"/>
+      <c r="E4" s="17"/>
+      <c r="F4" s="17"/>
     </row>
     <row r="6" spans="1:6" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="1" t="s">
+      <c r="A6" s="13" t="s">
         <v>165</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="B6" s="13" t="s">
         <v>97</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="C6" s="13" t="s">
         <v>166</v>
       </c>
-      <c r="D6" s="1" t="s">
+      <c r="D6" s="13" t="s">
         <v>167</v>
       </c>
-      <c r="E6" s="1" t="s">
+      <c r="E6" s="13" t="s">
         <v>168</v>
       </c>
-      <c r="F6" s="1" t="s">
+      <c r="F6" s="13" t="s">
         <v>169</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="7" t="s">
+      <c r="A7" s="14" t="s">
         <v>170</v>
       </c>
-      <c r="B7" s="7" t="s">
+      <c r="B7" s="14" t="s">
         <v>107</v>
       </c>
-      <c r="C7" s="7" t="s">
+      <c r="C7" s="14" t="s">
         <v>171</v>
       </c>
-      <c r="D7" s="7" t="s">
+      <c r="D7" s="14" t="s">
         <v>172</v>
       </c>
-      <c r="E7" s="7" t="s">
+      <c r="E7" s="14" t="s">
         <v>173</v>
       </c>
-      <c r="F7" s="7" t="s">
+      <c r="F7" s="14" t="s">
         <v>174</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="7" t="s">
+      <c r="A8" s="14" t="s">
         <v>175</v>
       </c>
-      <c r="B8" s="7" t="s">
+      <c r="B8" s="14" t="s">
         <v>116</v>
       </c>
-      <c r="C8" s="7" t="s">
+      <c r="C8" s="14" t="s">
         <v>176</v>
       </c>
-      <c r="D8" s="7" t="s">
+      <c r="D8" s="14" t="s">
         <v>172</v>
       </c>
-      <c r="E8" s="7" t="s">
+      <c r="E8" s="14" t="s">
         <v>90</v>
       </c>
-      <c r="F8" s="7" t="s">
+      <c r="F8" s="14" t="s">
         <v>90</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="7" t="s">
+      <c r="A9" s="14" t="s">
         <v>177</v>
       </c>
-      <c r="B9" s="7" t="s">
+      <c r="B9" s="14" t="s">
         <v>125</v>
       </c>
-      <c r="C9" s="7" t="s">
+      <c r="C9" s="14" t="s">
         <v>178</v>
       </c>
-      <c r="D9" s="7" t="s">
+      <c r="D9" s="14" t="s">
         <v>172</v>
       </c>
-      <c r="E9" s="7" t="s">
+      <c r="E9" s="14" t="s">
         <v>179</v>
       </c>
-      <c r="F9" s="7" t="s">
+      <c r="F9" s="14" t="s">
         <v>180</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="7" t="s">
+      <c r="A10" s="14" t="s">
         <v>181</v>
       </c>
-      <c r="B10" s="7" t="s">
+      <c r="B10" s="14" t="s">
         <v>136</v>
       </c>
-      <c r="C10" s="7" t="s">
+      <c r="C10" s="14" t="s">
         <v>182</v>
       </c>
-      <c r="D10" s="7" t="s">
+      <c r="D10" s="14" t="s">
         <v>172</v>
       </c>
-      <c r="E10" s="7" t="s">
+      <c r="E10" s="14" t="s">
         <v>183</v>
       </c>
-      <c r="F10" s="7" t="s">
+      <c r="F10" s="14" t="s">
         <v>184</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="7" t="s">
+      <c r="A11" s="14" t="s">
         <v>185</v>
       </c>
-      <c r="B11" s="7" t="s">
+      <c r="B11" s="14" t="s">
         <v>136</v>
       </c>
-      <c r="C11" s="7" t="s">
+      <c r="C11" s="14" t="s">
         <v>186</v>
       </c>
-      <c r="D11" s="7" t="s">
+      <c r="D11" s="14" t="s">
         <v>172</v>
       </c>
-      <c r="E11" s="7" t="s">
+      <c r="E11" s="14" t="s">
         <v>90</v>
       </c>
-      <c r="F11" s="7" t="s">
+      <c r="F11" s="14" t="s">
         <v>90</v>
       </c>
     </row>
@@ -4161,256 +4192,256 @@
   <dimension ref="A1:F30"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="22" style="4" customWidth="1"/>
-    <col min="2" max="2" width="44" style="4" customWidth="1"/>
-    <col min="3" max="4" width="14" style="4" customWidth="1"/>
-    <col min="5" max="5" width="20" style="4" customWidth="1"/>
-    <col min="6" max="6" width="14" style="4" customWidth="1"/>
-    <col min="7" max="16384" width="8.83203125" style="4"/>
+    <col min="1" max="1" width="22" style="15" customWidth="1"/>
+    <col min="2" max="2" width="44" style="15" customWidth="1"/>
+    <col min="3" max="4" width="14" style="15" customWidth="1"/>
+    <col min="5" max="5" width="20" style="15" customWidth="1"/>
+    <col min="6" max="6" width="14" style="15" customWidth="1"/>
+    <col min="7" max="16384" width="8.83203125" style="2"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="21" x14ac:dyDescent="0.2">
-      <c r="A1" s="8" t="s">
+      <c r="A1" s="16" t="s">
         <v>10</v>
       </c>
-      <c r="B1" s="3"/>
-      <c r="C1" s="3"/>
-      <c r="D1" s="3"/>
-      <c r="E1" s="3"/>
-      <c r="F1" s="3"/>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="17"/>
+      <c r="F1" s="17"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A2" s="5" t="s">
+      <c r="A2" s="18" t="s">
         <v>187</v>
       </c>
-      <c r="B2" s="3"/>
-      <c r="C2" s="3"/>
-      <c r="D2" s="3"/>
-      <c r="E2" s="3"/>
-      <c r="F2" s="3"/>
+      <c r="B2" s="17"/>
+      <c r="C2" s="17"/>
+      <c r="D2" s="17"/>
+      <c r="E2" s="17"/>
+      <c r="F2" s="17"/>
     </row>
     <row r="4" spans="1:6" ht="45" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="9" t="s">
+      <c r="A4" s="19" t="s">
         <v>188</v>
       </c>
-      <c r="B4" s="3"/>
-      <c r="C4" s="3"/>
-      <c r="D4" s="3"/>
-      <c r="E4" s="3"/>
-      <c r="F4" s="3"/>
+      <c r="B4" s="17"/>
+      <c r="C4" s="17"/>
+      <c r="D4" s="17"/>
+      <c r="E4" s="17"/>
+      <c r="F4" s="17"/>
     </row>
     <row r="6" spans="1:6" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="1" t="s">
+      <c r="A6" s="13" t="s">
         <v>189</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="B6" s="13" t="s">
         <v>190</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="C6" s="13" t="s">
         <v>191</v>
       </c>
-      <c r="D6" s="1" t="s">
+      <c r="D6" s="13" t="s">
         <v>167</v>
       </c>
-      <c r="E6" s="1" t="s">
+      <c r="E6" s="13" t="s">
         <v>192</v>
       </c>
-      <c r="F6" s="1" t="s">
+      <c r="F6" s="13" t="s">
         <v>97</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="7" t="s">
+      <c r="A7" s="14" t="s">
         <v>193</v>
       </c>
-      <c r="B7" s="7" t="s">
+      <c r="B7" s="14" t="s">
         <v>194</v>
       </c>
-      <c r="C7" s="7" t="s">
+      <c r="C7" s="14" t="s">
         <v>113</v>
       </c>
-      <c r="D7" s="7" t="s">
+      <c r="D7" s="14" t="s">
         <v>195</v>
       </c>
-      <c r="E7" s="7" t="s">
+      <c r="E7" s="14" t="s">
         <v>196</v>
       </c>
-      <c r="F7" s="7" t="s">
+      <c r="F7" s="14" t="s">
         <v>107</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="7" t="s">
+      <c r="A8" s="14" t="s">
         <v>197</v>
       </c>
-      <c r="B8" s="7" t="s">
+      <c r="B8" s="14" t="s">
         <v>194</v>
       </c>
-      <c r="C8" s="7" t="s">
+      <c r="C8" s="14" t="s">
         <v>198</v>
       </c>
-      <c r="D8" s="7" t="s">
+      <c r="D8" s="14" t="s">
         <v>199</v>
       </c>
-      <c r="E8" s="7" t="s">
+      <c r="E8" s="14" t="s">
         <v>200</v>
       </c>
-      <c r="F8" s="7" t="s">
+      <c r="F8" s="14" t="s">
         <v>116</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="7" t="s">
+      <c r="A9" s="14" t="s">
         <v>201</v>
       </c>
-      <c r="B9" s="7" t="s">
+      <c r="B9" s="14" t="s">
         <v>202</v>
       </c>
-      <c r="C9" s="7" t="s">
+      <c r="C9" s="14" t="s">
         <v>203</v>
       </c>
-      <c r="D9" s="7" t="s">
+      <c r="D9" s="14" t="s">
         <v>204</v>
       </c>
-      <c r="E9" s="7" t="s">
+      <c r="E9" s="14" t="s">
         <v>205</v>
       </c>
-      <c r="F9" s="7" t="s">
+      <c r="F9" s="14" t="s">
         <v>136</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="7" t="s">
+      <c r="A10" s="14" t="s">
         <v>206</v>
       </c>
-      <c r="B10" s="7" t="s">
+      <c r="B10" s="14" t="s">
         <v>207</v>
       </c>
-      <c r="C10" s="7" t="s">
+      <c r="C10" s="14" t="s">
         <v>113</v>
       </c>
-      <c r="D10" s="7" t="s">
+      <c r="D10" s="14" t="s">
         <v>195</v>
       </c>
-      <c r="E10" s="7" t="s">
+      <c r="E10" s="14" t="s">
         <v>196</v>
       </c>
-      <c r="F10" s="7" t="s">
+      <c r="F10" s="14" t="s">
         <v>125</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="7" t="s">
+      <c r="A11" s="14" t="s">
         <v>208</v>
       </c>
-      <c r="B11" s="7" t="s">
+      <c r="B11" s="14" t="s">
         <v>209</v>
       </c>
-      <c r="C11" s="7" t="s">
+      <c r="C11" s="14" t="s">
         <v>113</v>
       </c>
-      <c r="D11" s="7" t="s">
+      <c r="D11" s="14" t="s">
         <v>199</v>
       </c>
-      <c r="E11" s="7" t="s">
+      <c r="E11" s="14" t="s">
         <v>196</v>
       </c>
-      <c r="F11" s="7" t="s">
+      <c r="F11" s="14" t="s">
         <v>130</v>
       </c>
     </row>
     <row r="14" spans="1:6" ht="17" x14ac:dyDescent="0.2">
-      <c r="A14" s="10" t="s">
+      <c r="A14" s="20" t="s">
         <v>210</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A15" s="11" t="s">
+      <c r="A15" s="21" t="s">
         <v>211</v>
       </c>
     </row>
     <row r="17" spans="1:2" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="1" t="s">
+      <c r="A17" s="13" t="s">
         <v>212</v>
       </c>
-      <c r="B17" s="1" t="s">
+      <c r="B17" s="13" t="s">
         <v>213</v>
       </c>
     </row>
     <row r="18" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="7" t="s">
+      <c r="A18" s="14" t="s">
         <v>194</v>
       </c>
-      <c r="B18" s="7" t="s">
+      <c r="B18" s="14" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="19" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="7" t="s">
+      <c r="A19" s="14" t="s">
         <v>214</v>
       </c>
-      <c r="B19" s="7" t="s">
+      <c r="B19" s="14" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="20" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="7" t="s">
+      <c r="A20" s="14" t="s">
         <v>215</v>
       </c>
-      <c r="B20" s="7" t="s">
+      <c r="B20" s="14" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="21" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="7" t="s">
+      <c r="A21" s="14" t="s">
         <v>209</v>
       </c>
-      <c r="B21" s="7" t="s">
+      <c r="B21" s="14" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="22" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="7" t="s">
+      <c r="A22" s="14" t="s">
         <v>216</v>
       </c>
-      <c r="B22" s="7" t="s">
+      <c r="B22" s="14" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="25" spans="1:2" ht="17" x14ac:dyDescent="0.2">
-      <c r="A25" s="10" t="s">
+      <c r="A25" s="20" t="s">
         <v>217</v>
       </c>
     </row>
     <row r="27" spans="1:2" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="1" t="s">
+      <c r="A27" s="13" t="s">
         <v>218</v>
       </c>
-      <c r="B27" s="1" t="s">
+      <c r="B27" s="13" t="s">
         <v>219</v>
       </c>
     </row>
     <row r="28" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A28" s="7" t="s">
+      <c r="A28" s="14" t="s">
         <v>220</v>
       </c>
-      <c r="B28" s="7" t="s">
+      <c r="B28" s="14" t="s">
         <v>221</v>
       </c>
     </row>
     <row r="29" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A29" s="7" t="s">
+      <c r="A29" s="14" t="s">
         <v>222</v>
       </c>
-      <c r="B29" s="7" t="s">
+      <c r="B29" s="14" t="s">
         <v>223</v>
       </c>
     </row>
     <row r="30" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A30" s="7" t="s">
+      <c r="A30" s="14" t="s">
         <v>224</v>
       </c>
-      <c r="B30" s="7" t="s">
+      <c r="B30" s="14" t="s">
         <v>225</v>
       </c>
     </row>
@@ -4432,261 +4463,261 @@
   <dimension ref="A1:F16"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="14" style="4" customWidth="1"/>
-    <col min="2" max="2" width="34" style="4" customWidth="1"/>
-    <col min="3" max="4" width="14" style="4" customWidth="1"/>
-    <col min="5" max="5" width="12" style="4" customWidth="1"/>
-    <col min="6" max="6" width="34" style="4" customWidth="1"/>
-    <col min="7" max="16384" width="8.83203125" style="4"/>
+    <col min="1" max="1" width="14" style="15" customWidth="1"/>
+    <col min="2" max="2" width="34" style="15" customWidth="1"/>
+    <col min="3" max="4" width="14" style="15" customWidth="1"/>
+    <col min="5" max="5" width="12" style="15" customWidth="1"/>
+    <col min="6" max="6" width="34" style="15" customWidth="1"/>
+    <col min="7" max="16384" width="8.83203125" style="2"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="21" x14ac:dyDescent="0.2">
-      <c r="A1" s="8" t="s">
+      <c r="A1" s="16" t="s">
         <v>12</v>
       </c>
-      <c r="B1" s="3"/>
-      <c r="C1" s="3"/>
-      <c r="D1" s="3"/>
-      <c r="E1" s="3"/>
-      <c r="F1" s="3"/>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="17"/>
+      <c r="F1" s="17"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A2" s="5" t="s">
+      <c r="A2" s="18" t="s">
         <v>226</v>
       </c>
-      <c r="B2" s="3"/>
-      <c r="C2" s="3"/>
-      <c r="D2" s="3"/>
-      <c r="E2" s="3"/>
-      <c r="F2" s="3"/>
+      <c r="B2" s="17"/>
+      <c r="C2" s="17"/>
+      <c r="D2" s="17"/>
+      <c r="E2" s="17"/>
+      <c r="F2" s="17"/>
     </row>
     <row r="4" spans="1:6" ht="45" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="9" t="s">
+      <c r="A4" s="19" t="s">
         <v>227</v>
       </c>
-      <c r="B4" s="3"/>
-      <c r="C4" s="3"/>
-      <c r="D4" s="3"/>
-      <c r="E4" s="3"/>
-      <c r="F4" s="3"/>
+      <c r="B4" s="17"/>
+      <c r="C4" s="17"/>
+      <c r="D4" s="17"/>
+      <c r="E4" s="17"/>
+      <c r="F4" s="17"/>
     </row>
     <row r="6" spans="1:6" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="1" t="s">
+      <c r="A6" s="13" t="s">
         <v>228</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="B6" s="13" t="s">
         <v>229</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="C6" s="13" t="s">
         <v>230</v>
       </c>
-      <c r="D6" s="1" t="s">
+      <c r="D6" s="13" t="s">
         <v>167</v>
       </c>
-      <c r="E6" s="1" t="s">
+      <c r="E6" s="13" t="s">
         <v>231</v>
       </c>
-      <c r="F6" s="1" t="s">
+      <c r="F6" s="13" t="s">
         <v>232</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="7" t="s">
+      <c r="A7" s="14" t="s">
         <v>233</v>
       </c>
-      <c r="B7" s="7" t="s">
+      <c r="B7" s="14" t="s">
         <v>234</v>
       </c>
-      <c r="C7" s="7" t="s">
+      <c r="C7" s="14" t="s">
         <v>235</v>
       </c>
-      <c r="D7" s="7" t="s">
+      <c r="D7" s="14" t="s">
         <v>204</v>
       </c>
-      <c r="E7" s="7" t="s">
+      <c r="E7" s="14" t="s">
         <v>114</v>
       </c>
-      <c r="F7" s="7" t="s">
+      <c r="F7" s="14" t="s">
         <v>236</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="7" t="s">
+      <c r="A8" s="14" t="s">
         <v>237</v>
       </c>
-      <c r="B8" s="7" t="s">
+      <c r="B8" s="14" t="s">
         <v>238</v>
       </c>
-      <c r="C8" s="7" t="s">
+      <c r="C8" s="14" t="s">
         <v>235</v>
       </c>
-      <c r="D8" s="7" t="s">
+      <c r="D8" s="14" t="s">
         <v>204</v>
       </c>
-      <c r="E8" s="7" t="s">
+      <c r="E8" s="14" t="s">
         <v>123</v>
       </c>
-      <c r="F8" s="7" t="s">
+      <c r="F8" s="14" t="s">
         <v>236</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="7" t="s">
+      <c r="A9" s="14" t="s">
         <v>239</v>
       </c>
-      <c r="B9" s="7" t="s">
+      <c r="B9" s="14" t="s">
         <v>240</v>
       </c>
-      <c r="C9" s="7" t="s">
+      <c r="C9" s="14" t="s">
         <v>241</v>
       </c>
-      <c r="D9" s="7" t="s">
+      <c r="D9" s="14" t="s">
         <v>242</v>
       </c>
-      <c r="E9" s="7" t="s">
+      <c r="E9" s="14" t="s">
         <v>114</v>
       </c>
-      <c r="F9" s="7" t="s">
+      <c r="F9" s="14" t="s">
         <v>54</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="7" t="s">
+      <c r="A10" s="14" t="s">
         <v>243</v>
       </c>
-      <c r="B10" s="7" t="s">
+      <c r="B10" s="14" t="s">
         <v>244</v>
       </c>
-      <c r="C10" s="7" t="s">
+      <c r="C10" s="14" t="s">
         <v>235</v>
       </c>
-      <c r="D10" s="7" t="s">
+      <c r="D10" s="14" t="s">
         <v>245</v>
       </c>
-      <c r="E10" s="7" t="s">
+      <c r="E10" s="14" t="s">
         <v>114</v>
       </c>
-      <c r="F10" s="7" t="s">
+      <c r="F10" s="14" t="s">
         <v>54</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="7" t="s">
+      <c r="A11" s="14" t="s">
         <v>246</v>
       </c>
-      <c r="B11" s="7" t="s">
+      <c r="B11" s="14" t="s">
         <v>247</v>
       </c>
-      <c r="C11" s="7" t="s">
+      <c r="C11" s="14" t="s">
         <v>241</v>
       </c>
-      <c r="D11" s="7" t="s">
+      <c r="D11" s="14" t="s">
         <v>245</v>
       </c>
-      <c r="E11" s="7" t="s">
+      <c r="E11" s="14" t="s">
         <v>123</v>
       </c>
-      <c r="F11" s="7" t="s">
+      <c r="F11" s="14" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="12" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="7" t="s">
+      <c r="A12" s="14" t="s">
         <v>248</v>
       </c>
-      <c r="B12" s="7" t="s">
+      <c r="B12" s="14" t="s">
         <v>249</v>
       </c>
-      <c r="C12" s="7" t="s">
+      <c r="C12" s="14" t="s">
         <v>250</v>
       </c>
-      <c r="D12" s="7" t="s">
+      <c r="D12" s="14" t="s">
         <v>204</v>
       </c>
-      <c r="E12" s="7" t="s">
+      <c r="E12" s="14" t="s">
         <v>114</v>
       </c>
-      <c r="F12" s="7" t="s">
+      <c r="F12" s="14" t="s">
         <v>236</v>
       </c>
     </row>
     <row r="13" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="7" t="s">
+      <c r="A13" s="14" t="s">
         <v>251</v>
       </c>
-      <c r="B13" s="7" t="s">
+      <c r="B13" s="14" t="s">
         <v>252</v>
       </c>
-      <c r="C13" s="7" t="s">
+      <c r="C13" s="14" t="s">
         <v>250</v>
       </c>
-      <c r="D13" s="7" t="s">
+      <c r="D13" s="14" t="s">
         <v>242</v>
       </c>
-      <c r="E13" s="7" t="s">
+      <c r="E13" s="14" t="s">
         <v>123</v>
       </c>
-      <c r="F13" s="7" t="s">
+      <c r="F13" s="14" t="s">
         <v>54</v>
       </c>
     </row>
     <row r="14" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="7" t="s">
+      <c r="A14" s="14" t="s">
         <v>253</v>
       </c>
-      <c r="B14" s="7" t="s">
+      <c r="B14" s="14" t="s">
         <v>254</v>
       </c>
-      <c r="C14" s="7" t="s">
+      <c r="C14" s="14" t="s">
         <v>235</v>
       </c>
-      <c r="D14" s="7" t="s">
+      <c r="D14" s="14" t="s">
         <v>255</v>
       </c>
-      <c r="E14" s="7" t="s">
+      <c r="E14" s="14" t="s">
         <v>114</v>
       </c>
-      <c r="F14" s="7" t="s">
+      <c r="F14" s="14" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="15" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="7" t="s">
+      <c r="A15" s="14" t="s">
         <v>256</v>
       </c>
-      <c r="B15" s="7" t="s">
+      <c r="B15" s="14" t="s">
         <v>257</v>
       </c>
-      <c r="C15" s="7" t="s">
+      <c r="C15" s="14" t="s">
         <v>241</v>
       </c>
-      <c r="D15" s="7" t="s">
+      <c r="D15" s="14" t="s">
         <v>204</v>
       </c>
-      <c r="E15" s="7" t="s">
+      <c r="E15" s="14" t="s">
         <v>114</v>
       </c>
-      <c r="F15" s="7" t="s">
+      <c r="F15" s="14" t="s">
         <v>236</v>
       </c>
     </row>
     <row r="16" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="7" t="s">
+      <c r="A16" s="14" t="s">
         <v>258</v>
       </c>
-      <c r="B16" s="7" t="s">
+      <c r="B16" s="14" t="s">
         <v>259</v>
       </c>
-      <c r="C16" s="7" t="s">
+      <c r="C16" s="14" t="s">
         <v>250</v>
       </c>
-      <c r="D16" s="7" t="s">
+      <c r="D16" s="14" t="s">
         <v>245</v>
       </c>
-      <c r="E16" s="7" t="s">
+      <c r="E16" s="14" t="s">
         <v>114</v>
       </c>
-      <c r="F16" s="7" t="s">
+      <c r="F16" s="14" t="s">
         <v>54</v>
       </c>
     </row>
@@ -4708,272 +4739,272 @@
   <dimension ref="A1:I21"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="14" style="4" customWidth="1"/>
-    <col min="2" max="2" width="90" style="4" customWidth="1"/>
-    <col min="3" max="3" width="14" style="4" customWidth="1"/>
-    <col min="4" max="4" width="20" style="4" customWidth="1"/>
-    <col min="5" max="5" width="14" style="4" customWidth="1"/>
-    <col min="6" max="6" width="12" style="4" customWidth="1"/>
-    <col min="7" max="7" width="18" style="4" customWidth="1"/>
-    <col min="8" max="8" width="16" style="4" customWidth="1"/>
-    <col min="9" max="9" width="14" style="4" customWidth="1"/>
-    <col min="10" max="16384" width="8.83203125" style="4"/>
+    <col min="1" max="1" width="14" style="15" customWidth="1"/>
+    <col min="2" max="2" width="90" style="15" customWidth="1"/>
+    <col min="3" max="3" width="14" style="15" customWidth="1"/>
+    <col min="4" max="4" width="20" style="15" customWidth="1"/>
+    <col min="5" max="5" width="14" style="15" customWidth="1"/>
+    <col min="6" max="6" width="12" style="15" customWidth="1"/>
+    <col min="7" max="7" width="18" style="15" customWidth="1"/>
+    <col min="8" max="8" width="16" style="15" customWidth="1"/>
+    <col min="9" max="9" width="14" style="15" customWidth="1"/>
+    <col min="10" max="16384" width="8.83203125" style="2"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="21" x14ac:dyDescent="0.2">
-      <c r="A1" s="8" t="s">
+      <c r="A1" s="16" t="s">
         <v>14</v>
       </c>
-      <c r="B1" s="3"/>
-      <c r="C1" s="3"/>
-      <c r="D1" s="3"/>
-      <c r="E1" s="3"/>
-      <c r="F1" s="3"/>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="17"/>
+      <c r="F1" s="17"/>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A2" s="5" t="s">
+      <c r="A2" s="18" t="s">
         <v>260</v>
       </c>
-      <c r="B2" s="3"/>
-      <c r="C2" s="3"/>
-      <c r="D2" s="3"/>
-      <c r="E2" s="3"/>
-      <c r="F2" s="3"/>
+      <c r="B2" s="17"/>
+      <c r="C2" s="17"/>
+      <c r="D2" s="17"/>
+      <c r="E2" s="17"/>
+      <c r="F2" s="17"/>
     </row>
     <row r="4" spans="1:9" ht="45" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="9" t="s">
+      <c r="A4" s="19" t="s">
         <v>261</v>
       </c>
-      <c r="B4" s="3"/>
-      <c r="C4" s="3"/>
-      <c r="D4" s="3"/>
-      <c r="E4" s="3"/>
-      <c r="F4" s="3"/>
+      <c r="B4" s="17"/>
+      <c r="C4" s="17"/>
+      <c r="D4" s="17"/>
+      <c r="E4" s="17"/>
+      <c r="F4" s="17"/>
     </row>
     <row r="6" spans="1:9" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="1" t="s">
+      <c r="A6" s="13" t="s">
         <v>262</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="B6" s="13" t="s">
         <v>97</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="C6" s="13" t="s">
         <v>167</v>
       </c>
-      <c r="D6" s="1" t="s">
+      <c r="D6" s="13" t="s">
         <v>263</v>
       </c>
-      <c r="E6" s="1" t="s">
+      <c r="E6" s="13" t="s">
         <v>264</v>
       </c>
-      <c r="F6" s="1" t="s">
+      <c r="F6" s="13" t="s">
         <v>265</v>
       </c>
-      <c r="G6" s="1" t="s">
+      <c r="G6" s="13" t="s">
         <v>266</v>
       </c>
-      <c r="H6" s="1" t="s">
+      <c r="H6" s="13" t="s">
         <v>267</v>
       </c>
-      <c r="I6" s="1" t="s">
+      <c r="I6" s="13" t="s">
         <v>268</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="7" t="s">
+      <c r="A7" s="14" t="s">
         <v>269</v>
       </c>
-      <c r="B7" s="7" t="s">
+      <c r="B7" s="14" t="s">
         <v>107</v>
       </c>
-      <c r="C7" s="7" t="s">
+      <c r="C7" s="14" t="s">
         <v>270</v>
       </c>
-      <c r="D7" s="7" t="s">
+      <c r="D7" s="14" t="s">
         <v>271</v>
       </c>
-      <c r="E7" s="7" t="s">
+      <c r="E7" s="14" t="s">
         <v>272</v>
       </c>
-      <c r="F7" s="7" t="s">
+      <c r="F7" s="14" t="s">
         <v>273</v>
       </c>
-      <c r="G7" s="7" t="s">
+      <c r="G7" s="14" t="s">
         <v>274</v>
       </c>
-      <c r="H7" s="7" t="s">
+      <c r="H7" s="14" t="s">
         <v>90</v>
       </c>
-      <c r="I7" s="7">
+      <c r="I7" s="14">
         <v>24</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="7" t="s">
+      <c r="A8" s="14" t="s">
         <v>275</v>
       </c>
-      <c r="B8" s="7" t="s">
+      <c r="B8" s="14" t="s">
         <v>125</v>
       </c>
-      <c r="C8" s="7" t="s">
+      <c r="C8" s="14" t="s">
         <v>255</v>
       </c>
-      <c r="D8" s="7" t="s">
+      <c r="D8" s="14" t="s">
         <v>276</v>
       </c>
-      <c r="E8" s="7" t="s">
+      <c r="E8" s="14" t="s">
         <v>277</v>
       </c>
-      <c r="F8" s="7" t="s">
+      <c r="F8" s="14" t="s">
         <v>278</v>
       </c>
-      <c r="G8" s="7" t="s">
+      <c r="G8" s="14" t="s">
         <v>279</v>
       </c>
-      <c r="H8" s="7" t="s">
+      <c r="H8" s="14" t="s">
         <v>280</v>
       </c>
-      <c r="I8" s="7">
+      <c r="I8" s="14">
         <v>24</v>
       </c>
     </row>
     <row r="9" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="7" t="s">
+      <c r="A9" s="14" t="s">
         <v>281</v>
       </c>
-      <c r="B9" s="7" t="s">
+      <c r="B9" s="14" t="s">
         <v>116</v>
       </c>
-      <c r="C9" s="7" t="s">
+      <c r="C9" s="14" t="s">
         <v>282</v>
       </c>
-      <c r="D9" s="7" t="s">
+      <c r="D9" s="14" t="s">
         <v>271</v>
       </c>
-      <c r="E9" s="7" t="s">
+      <c r="E9" s="14" t="s">
         <v>283</v>
       </c>
-      <c r="F9" s="7" t="s">
+      <c r="F9" s="14" t="s">
         <v>284</v>
       </c>
-      <c r="G9" s="7" t="s">
+      <c r="G9" s="14" t="s">
         <v>279</v>
       </c>
-      <c r="H9" s="7" t="s">
+      <c r="H9" s="14" t="s">
         <v>280</v>
       </c>
-      <c r="I9" s="7">
+      <c r="I9" s="14">
         <v>48</v>
       </c>
     </row>
     <row r="10" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="7" t="s">
+      <c r="A10" s="14" t="s">
         <v>285</v>
       </c>
-      <c r="B10" s="7" t="s">
+      <c r="B10" s="14" t="s">
         <v>130</v>
       </c>
-      <c r="C10" s="7" t="s">
+      <c r="C10" s="14" t="s">
         <v>255</v>
       </c>
-      <c r="D10" s="7" t="s">
+      <c r="D10" s="14" t="s">
         <v>286</v>
       </c>
-      <c r="E10" s="7" t="s">
+      <c r="E10" s="14" t="s">
         <v>287</v>
       </c>
-      <c r="F10" s="7" t="s">
+      <c r="F10" s="14" t="s">
         <v>273</v>
       </c>
-      <c r="G10" s="7" t="s">
+      <c r="G10" s="14" t="s">
         <v>279</v>
       </c>
-      <c r="H10" s="7" t="s">
+      <c r="H10" s="14" t="s">
         <v>280</v>
       </c>
-      <c r="I10" s="7">
+      <c r="I10" s="14">
         <v>24</v>
       </c>
     </row>
     <row r="11" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="7" t="s">
+      <c r="A11" s="14" t="s">
         <v>288</v>
       </c>
-      <c r="B11" s="7" t="s">
+      <c r="B11" s="14" t="s">
         <v>136</v>
       </c>
-      <c r="C11" s="7" t="s">
+      <c r="C11" s="14" t="s">
         <v>242</v>
       </c>
-      <c r="D11" s="7" t="s">
+      <c r="D11" s="14" t="s">
         <v>289</v>
       </c>
-      <c r="E11" s="7" t="s">
+      <c r="E11" s="14" t="s">
         <v>290</v>
       </c>
-      <c r="F11" s="7" t="s">
+      <c r="F11" s="14" t="s">
         <v>291</v>
       </c>
-      <c r="G11" s="7" t="s">
+      <c r="G11" s="14" t="s">
         <v>279</v>
       </c>
-      <c r="H11" s="7" t="s">
+      <c r="H11" s="14" t="s">
         <v>280</v>
       </c>
-      <c r="I11" s="7">
+      <c r="I11" s="14">
         <v>24</v>
       </c>
     </row>
     <row r="14" spans="1:9" ht="17" x14ac:dyDescent="0.2">
-      <c r="A14" s="10" t="s">
+      <c r="A14" s="20" t="s">
         <v>292</v>
       </c>
     </row>
     <row r="16" spans="1:9" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="1" t="s">
+      <c r="A16" s="13" t="s">
         <v>293</v>
       </c>
-      <c r="B16" s="1" t="s">
+      <c r="B16" s="13" t="s">
         <v>294</v>
       </c>
     </row>
     <row r="17" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="7" t="s">
+      <c r="A17" s="14" t="s">
         <v>269</v>
       </c>
-      <c r="B17" s="7" t="s">
+      <c r="B17" s="14" t="s">
         <v>295</v>
       </c>
     </row>
     <row r="18" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="7" t="s">
+      <c r="A18" s="14" t="s">
         <v>275</v>
       </c>
-      <c r="B18" s="7" t="s">
+      <c r="B18" s="14" t="s">
         <v>296</v>
       </c>
     </row>
     <row r="19" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="7" t="s">
+      <c r="A19" s="14" t="s">
         <v>281</v>
       </c>
-      <c r="B19" s="7" t="s">
+      <c r="B19" s="14" t="s">
         <v>297</v>
       </c>
     </row>
     <row r="20" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="7" t="s">
+      <c r="A20" s="14" t="s">
         <v>285</v>
       </c>
-      <c r="B20" s="7" t="s">
+      <c r="B20" s="14" t="s">
         <v>298</v>
       </c>
     </row>
     <row r="21" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="7" t="s">
+      <c r="A21" s="14" t="s">
         <v>288</v>
       </c>
-      <c r="B21" s="7" t="s">
+      <c r="B21" s="14" t="s">
         <v>299</v>
       </c>
     </row>
@@ -4995,126 +5026,126 @@
   <dimension ref="A1:F10"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="16" style="4" customWidth="1"/>
-    <col min="2" max="2" width="14" style="4" customWidth="1"/>
-    <col min="3" max="3" width="12" style="4" customWidth="1"/>
-    <col min="4" max="4" width="26" style="4" customWidth="1"/>
-    <col min="5" max="5" width="55" style="4" customWidth="1"/>
-    <col min="6" max="16384" width="8.83203125" style="4"/>
+    <col min="1" max="1" width="16" style="15" customWidth="1"/>
+    <col min="2" max="2" width="14" style="15" customWidth="1"/>
+    <col min="3" max="3" width="12" style="15" customWidth="1"/>
+    <col min="4" max="4" width="26" style="15" customWidth="1"/>
+    <col min="5" max="5" width="55" style="15" customWidth="1"/>
+    <col min="6" max="16384" width="8.83203125" style="2"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="21" x14ac:dyDescent="0.2">
-      <c r="A1" s="8" t="s">
+      <c r="A1" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="B1" s="3"/>
-      <c r="C1" s="3"/>
-      <c r="D1" s="3"/>
-      <c r="E1" s="3"/>
-      <c r="F1" s="3"/>
+      <c r="B1" s="6"/>
+      <c r="C1" s="6"/>
+      <c r="D1" s="6"/>
+      <c r="E1" s="6"/>
+      <c r="F1" s="6"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" s="5" t="s">
         <v>300</v>
       </c>
-      <c r="B2" s="3"/>
-      <c r="C2" s="3"/>
-      <c r="D2" s="3"/>
-      <c r="E2" s="3"/>
-      <c r="F2" s="3"/>
+      <c r="B2" s="6"/>
+      <c r="C2" s="6"/>
+      <c r="D2" s="6"/>
+      <c r="E2" s="6"/>
+      <c r="F2" s="6"/>
     </row>
     <row r="4" spans="1:6" ht="45" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="9" t="s">
+      <c r="A4" s="8" t="s">
         <v>301</v>
       </c>
-      <c r="B4" s="3"/>
-      <c r="C4" s="3"/>
-      <c r="D4" s="3"/>
-      <c r="E4" s="3"/>
-      <c r="F4" s="3"/>
+      <c r="B4" s="6"/>
+      <c r="C4" s="6"/>
+      <c r="D4" s="6"/>
+      <c r="E4" s="6"/>
+      <c r="F4" s="6"/>
     </row>
     <row r="6" spans="1:6" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="1" t="s">
+      <c r="A6" s="13" t="s">
         <v>302</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="B6" s="13" t="s">
         <v>97</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="C6" s="13" t="s">
         <v>167</v>
       </c>
-      <c r="D6" s="1" t="s">
+      <c r="D6" s="13" t="s">
         <v>303</v>
       </c>
-      <c r="E6" s="1" t="s">
+      <c r="E6" s="13" t="s">
         <v>304</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="7" t="s">
+      <c r="A7" s="14" t="s">
         <v>305</v>
       </c>
-      <c r="B7" s="7" t="s">
+      <c r="B7" s="14" t="s">
         <v>107</v>
       </c>
-      <c r="C7" s="7" t="s">
+      <c r="C7" s="14" t="s">
         <v>306</v>
       </c>
-      <c r="D7" s="7" t="s">
+      <c r="D7" s="14" t="s">
         <v>307</v>
       </c>
-      <c r="E7" s="7" t="s">
+      <c r="E7" s="14" t="s">
         <v>308</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="7" t="s">
+      <c r="A8" s="14" t="s">
         <v>309</v>
       </c>
-      <c r="B8" s="7" t="s">
+      <c r="B8" s="14" t="s">
         <v>125</v>
       </c>
-      <c r="C8" s="7" t="s">
+      <c r="C8" s="14" t="s">
         <v>306</v>
       </c>
-      <c r="D8" s="7" t="s">
+      <c r="D8" s="14" t="s">
         <v>310</v>
       </c>
-      <c r="E8" s="7" t="s">
+      <c r="E8" s="14" t="s">
         <v>311</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="7" t="s">
+      <c r="A9" s="14" t="s">
         <v>312</v>
       </c>
-      <c r="B9" s="7" t="s">
+      <c r="B9" s="14" t="s">
         <v>107</v>
       </c>
-      <c r="C9" s="7" t="s">
+      <c r="C9" s="14" t="s">
         <v>313</v>
       </c>
-      <c r="D9" s="7" t="s">
+      <c r="D9" s="14" t="s">
         <v>90</v>
       </c>
-      <c r="E9" s="7" t="s">
+      <c r="E9" s="14" t="s">
         <v>314</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="7" t="s">
+      <c r="A10" s="14" t="s">
         <v>315</v>
       </c>
-      <c r="B10" s="7" t="s">
+      <c r="B10" s="14" t="s">
         <v>116</v>
       </c>
-      <c r="C10" s="7" t="s">
+      <c r="C10" s="14" t="s">
         <v>306</v>
       </c>
-      <c r="D10" s="7" t="s">
+      <c r="D10" s="14" t="s">
         <v>316</v>
       </c>
-      <c r="E10" s="7" t="s">
+      <c r="E10" s="14" t="s">
         <v>317</v>
       </c>
     </row>
@@ -5136,82 +5167,82 @@
   <dimension ref="A1:F8"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="14" style="4" customWidth="1"/>
-    <col min="2" max="2" width="30" style="4" customWidth="1"/>
-    <col min="3" max="3" width="22" style="4" customWidth="1"/>
-    <col min="4" max="4" width="60" style="4" customWidth="1"/>
-    <col min="5" max="16384" width="8.83203125" style="4"/>
+    <col min="1" max="1" width="14" style="15" customWidth="1"/>
+    <col min="2" max="2" width="30" style="15" customWidth="1"/>
+    <col min="3" max="3" width="22" style="15" customWidth="1"/>
+    <col min="4" max="4" width="60" style="15" customWidth="1"/>
+    <col min="5" max="16384" width="8.83203125" style="2"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="21" x14ac:dyDescent="0.2">
-      <c r="A1" s="8" t="s">
+      <c r="A1" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="B1" s="3"/>
-      <c r="C1" s="3"/>
-      <c r="D1" s="3"/>
-      <c r="E1" s="3"/>
-      <c r="F1" s="3"/>
+      <c r="B1" s="6"/>
+      <c r="C1" s="6"/>
+      <c r="D1" s="6"/>
+      <c r="E1" s="6"/>
+      <c r="F1" s="6"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" s="5" t="s">
         <v>318</v>
       </c>
-      <c r="B2" s="3"/>
-      <c r="C2" s="3"/>
-      <c r="D2" s="3"/>
-      <c r="E2" s="3"/>
-      <c r="F2" s="3"/>
+      <c r="B2" s="6"/>
+      <c r="C2" s="6"/>
+      <c r="D2" s="6"/>
+      <c r="E2" s="6"/>
+      <c r="F2" s="6"/>
     </row>
     <row r="4" spans="1:6" ht="45" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="9" t="s">
+      <c r="A4" s="8" t="s">
         <v>319</v>
       </c>
-      <c r="B4" s="3"/>
-      <c r="C4" s="3"/>
-      <c r="D4" s="3"/>
-      <c r="E4" s="3"/>
-      <c r="F4" s="3"/>
+      <c r="B4" s="6"/>
+      <c r="C4" s="6"/>
+      <c r="D4" s="6"/>
+      <c r="E4" s="6"/>
+      <c r="F4" s="6"/>
     </row>
     <row r="6" spans="1:6" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="1" t="s">
+      <c r="A6" s="13" t="s">
         <v>320</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="B6" s="13" t="s">
         <v>321</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="C6" s="13" t="s">
         <v>322</v>
       </c>
-      <c r="D6" s="1" t="s">
+      <c r="D6" s="13" t="s">
         <v>323</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="7" t="s">
+      <c r="A7" s="14" t="s">
         <v>324</v>
       </c>
-      <c r="B7" s="7" t="s">
+      <c r="B7" s="14" t="s">
         <v>325</v>
       </c>
-      <c r="C7" s="7" t="s">
+      <c r="C7" s="14" t="s">
         <v>326</v>
       </c>
-      <c r="D7" s="7" t="s">
+      <c r="D7" s="14" t="s">
         <v>327</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="7" t="s">
+      <c r="A8" s="14" t="s">
         <v>328</v>
       </c>
-      <c r="B8" s="7" t="s">
+      <c r="B8" s="14" t="s">
         <v>170</v>
       </c>
-      <c r="C8" s="7" t="s">
+      <c r="C8" s="14" t="s">
         <v>329</v>
       </c>
-      <c r="D8" s="7" t="s">
+      <c r="D8" s="14" t="s">
         <v>330</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Remediate Customer 360 BRSD gaps; add session reference header
- Implement all previously Missing/Partial Customer 360 BRSD v3.1
  requirements: demographic/contact/address/billing edit drawers,
  account hierarchy drill-down, invoice download/print/resend,
  attachment status/filtering, interaction logging, and the BR-01
  identity verification gate (QID scan + ID-number match).
- Fix a BR-02 edit-access bypass and ticket/interaction data
  staleness found during independent re-verification of the above.
- Add a persistent header display of the Qnomy Ticket Number (Retail
  Agents/managers) and CTI Reference Number (Back-Office
  Agents/managers), gated by role, with a Finish -> Next Customer
  servicing workflow that never auto-advances the walk-in queue.
- Center, then reposition, the global search box in the topbar.
- Rebuild the BRSD audit workbook to reflect the remediated state.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/vfq-dxp-app/reference/VFQ_DXP_Test_Data_Reference.xlsx
+++ b/vfq-dxp-app/reference/VFQ_DXP_Test_Data_Reference.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/parithimalsaravanan/claude-projects/vfq/vfq-dxp-app/reference/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6EE90C55-6906-3144-9B04-627C2F7C9491}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8AE94B60-11BD-054A-A9E1-3EECAD795E72}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="21680" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="21680" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Start Here" sheetId="1" r:id="rId1"/>
@@ -1681,7 +1681,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -1770,6 +1770,12 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3899,6 +3905,7 @@
     <mergeCell ref="A4:F4"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="8" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
   <headerFooter>
     <oddFooter>&amp;L&amp;"Aptos"&amp;10 &amp;K000000_x000D_# Public</oddFooter>
   </headerFooter>
@@ -3943,12 +3950,12 @@
       <c r="E2" s="17"/>
       <c r="F2" s="17"/>
     </row>
-    <row r="4" spans="1:10" ht="60" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="20" t="s">
+    <row r="4" spans="1:10" ht="83" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="31" t="s">
         <v>2</v>
       </c>
       <c r="B4" s="17"/>
-      <c r="C4" s="18"/>
+      <c r="C4" s="32"/>
       <c r="D4" s="17"/>
       <c r="E4" s="17"/>
       <c r="F4" s="17"/>

</xml_diff>